<commit_message>
Add GitHub evidence links to manual API test results
</commit_message>
<xml_diff>
--- a/test-documentation/ServeRest_API_Test_Cases.xlsx
+++ b/test-documentation/ServeRest_API_Test_Cases.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="210">
   <si>
     <t>ServeRest API — Manual Test Cases</t>
   </si>
@@ -630,7 +630,7 @@
     <t>16 test runs  |  See Remarks for any test limitations</t>
   </si>
   <si>
-    <t>Actual results follow the same numbered checks as Expected. [E#] points to evidence files in column H.</t>
+    <t>Execution details are grouped by test case; every E# is a separate clickable screenshot.</t>
   </si>
   <si>
     <t>TEST RESULTS  |  MAN-001 TO MAN-016</t>
@@ -663,7 +663,7 @@
     <t>Test Status</t>
   </si>
   <si>
-    <t>Evidence</t>
+    <t>Evidence Link</t>
   </si>
   <si>
     <t>Remarks / Defect ID</t>
@@ -683,10 +683,6 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>E1. evidence/manual-api/user-management/TC-USER-001_CREATE_USER_REQUEST.png
-E2. evidence/manual-api/user-management/TC-USER-001_CREATE_USER_RESPONSE.png</t>
-  </si>
-  <si>
     <t>Created a test user and saved request/response screenshots.</t>
   </si>
   <si>
@@ -697,10 +693,6 @@
 2. Message was "Este email já está sendo usado". [E2]</t>
   </si>
   <si>
-    <t>E1. evidence/manual-api/user-management/TC-USER-002_DUPLICATE_EMAIL_REQUEST.png
-E2. evidence/manual-api/user-management/TC-USER-002_DUPLICATE_EMAIL_RESPONSE.png</t>
-  </si>
-  <si>
     <t>Used the same email as TC-USER-001. The API rejected the duplicate email.</t>
   </si>
   <si>
@@ -709,10 +701,6 @@
   <si>
     <t>1. HTTP response was 400 Bad Request. [E2]
 2. Email error was "email é obrigatório". [E2]</t>
-  </si>
-  <si>
-    <t>E1. evidence/manual-api/user-management/TC-USER-003_MISSING_EMAIL_REQUEST.png
-E2. evidence/manual-api/user-management/TC-USER-003_MISSING_EMAIL_RESPONSE.png</t>
   </si>
   <si>
     <t>Left out the email field (not an empty string). The API rejected the request.</t>
@@ -726,10 +714,6 @@
 3. Returned _id matched GdTunqRyBjbu2bJr. [E1, E2]</t>
   </si>
   <si>
-    <t>E1. evidence/manual-api/user-management/TC-USER-004_GET_USER_REQUEST.png
-E2. evidence/manual-api/user-management/TC-USER-004_GET_USER_RESPONSE.png</t>
-  </si>
-  <si>
     <t>Checked the same user ID created in TC-USER-001.</t>
   </si>
   <si>
@@ -739,10 +723,6 @@
     <t>1. HTTP response was 200 OK. [E2]
 2. Message was "Login realizado com sucesso". [E2]
 3. Authorization included a non-empty Bearer token; the value is redacted in public evidence. [E2]</t>
-  </si>
-  <si>
-    <t>E1. evidence/manual-api/authentication/TC-AUTH-001_VALID_LOGIN_REQUEST.png
-E2. evidence/manual-api/authentication/TC-AUTH-001_VALID_LOGIN_RESPONSE.png</t>
   </si>
   <si>
     <t>Created the test user first, then logged in. Redact Bearer tokens in screenshots.</t>
@@ -756,10 +736,6 @@
 3. The authorization field was absent. [E2]</t>
   </si>
   <si>
-    <t>E1. evidence/manual-api/authentication/TC-AUTH-002_INVALID_PASSWORD_REQUEST.png
-E2. evidence/manual-api/authentication/TC-AUTH-002_INVALID_PASSWORD_RESPONSE.png</t>
-  </si>
-  <si>
     <t>Valid login worked for this account. The incorrect password was rejected.</t>
   </si>
   <si>
@@ -769,11 +745,6 @@
     <t>1. GET /usuarios?email=... returned quantidade = 0 and usuarios = []. [E3]
 2. POST /login returned 401 Unauthorized; message was "Email e/ou senha inválidos". [E2]
 3. The authorization field was absent. [E2]</t>
-  </si>
-  <si>
-    <t>E1. evidence/manual-api/authentication/TC-AUTH-003_UNREGISTERED_EMAIL_REQUEST.png
-E2. evidence/manual-api/authentication/TC-AUTH-003_UNREGISTERED_EMAIL_RESPONSE.png
-E3. evidence/manual-api/authentication/CHECK_UNREGISTERED_EMAIL_RESPONSE.png</t>
   </si>
   <si>
     <t>Confirmed the email was not registered before testing. Login was rejected.</t>
@@ -787,10 +758,6 @@
 3. No authorization field or usable token was returned. [E2]</t>
   </si>
   <si>
-    <t>E1. evidence/manual-api/authentication/TC-AUTH-004_MISSING_EMAIL_REQUEST.png
-E2. evidence/manual-api/authentication/TC-AUTH-004_MISSING_EMAIL_RESPONSE.png</t>
-  </si>
-  <si>
     <t>Missing email was rejected and no token was issued. Exact status/message requirements still need confirmation.</t>
   </si>
   <si>
@@ -800,10 +767,6 @@
     <t>1. GET /produtos returned 200 OK. [E2]
 2. Response contained quantidade = 356 and a produtos array; inspected item included the required fields. [E2]
 3. Postman Console check showed produtos.length = 356, matching quantidade (console check reported in execution notes; no separately listed console screenshot).</t>
-  </si>
-  <si>
-    <t>E1. evidence/manual-api/products/TC-PROD-001_GET_PRODUCTS_REQUEST.png
-E2. evidence/manual-api/products/TC-PROD-001_GET_PRODUCTS_RESPONSE.png</t>
   </si>
   <si>
     <t>Public product data may change. Checked list count in Postman Console; no console screenshot saved.</t>
@@ -817,10 +780,6 @@
 3. Returned _id matched 2ReHn2QArWo1U7sa. [E1, E2]</t>
   </si>
   <si>
-    <t>E1. evidence/manual-api/products/TC-PROD-002_GET_PRODUCT_REQUEST.png
-E2. evidence/manual-api/products/TC-PROD-002_GET_PRODUCT_RESPONSE.png</t>
-  </si>
-  <si>
     <t>Used a product that existed at test time. Stock quantity of 0 does not affect this GET test.</t>
   </si>
   <si>
@@ -832,11 +791,6 @@
 3. Follow-up GET returned 200 OK; nome = "QA Mouse Test 20261023 001", preco = 470, descricao = "Mouse", quantidade = 381 and _id matched the create request. [E1, E3]</t>
   </si>
   <si>
-    <t>E1. evidence/manual-api/products/TC-PROD-003_CREATE_PRODUCT_REQUEST.png
-E2. evidence/manual-api/products/TC-PROD-003_CREATE_PRODUCT_RESPONSE.png
-E3. evidence/manual-api/products/CHECK_CREATED_PRODUCT_RESPONSE.png</t>
-  </si>
-  <si>
     <t>First attempt used a non-admin token (403). Retried with admin token and confirmed product creation. Hide secrets in screenshots.</t>
   </si>
   <si>
@@ -846,11 +800,6 @@
     <t>1. POST /produtos returned 400 Bad Request. [E2]
 2. Message was "Já existe produto com esse nome". [E2]
 3. GET /produtos?nome=... returned 200 OK and exactly one matching product, with the original setup _id. [E3]</t>
-  </si>
-  <si>
-    <t>E1. evidence/manual-api/products/TC-PROD-004_DUPLICATE_PRODUCT_REQUEST.png
-E2. evidence/manual-api/products/TC-PROD-004_DUPLICATE_PRODUCT_RESPONSE.png
-E3. evidence/manual-api/products/TC-PROD-004_VERIFY_NO_DUPLICATE_RESPONSE.png</t>
   </si>
   <si>
     <t>Created the product during setup. The API rejected another product with the same name.</t>
@@ -865,13 +814,6 @@
 4. Follow-up GET showed stock decreased from 5 to 3. [E4, E5]</t>
   </si>
   <si>
-    <t>E1. evidence/manual-api/cart/TC-CART-001_CREATE_CART_REQUEST.png
-E2. evidence/manual-api/cart/TC-CART-001_CREATE_CART_RESPONSE.png
-E3. evidence/manual-api/cart/TC-CART-001_VERIFY_CART_RESPONSE.png
-E4. evidence/manual-api/cart/TC-CART-001_STOCK_BEFORE.png
-E5. evidence/manual-api/cart/TC-CART-001_STOCK_AFTER.png</t>
-  </si>
-  <si>
     <t>Cart contained 2 items, total 198. Stock decreased from 5 to 3. Check screenshot paths before publishing.</t>
   </si>
   <si>
@@ -881,11 +823,6 @@
     <t>1. GET /carrinhos/0xcWZJaV4S2epqF8 returned 200 OK; existing cart contained product 8TFymQZ8RB52F4uD, quantity 2, total 198. [E1]
 2. POST /carrinhos with the same user token returned 400 Bad Request. [E3]
 3. Response message was "Não é permitido ter mais de 1 carrinho". [E3]</t>
-  </si>
-  <si>
-    <t>E1. evidence/manual-api/cart/TC-CART-002_EXISTING_CART_RESPONSE.png
-E2. evidence/manual-api/cart/TC-CART-002_SECOND_CART_REQUEST.png
-E3. evidence/manual-api/cart/TC-CART-002_SECOND_CART_RESPONSE.png</t>
   </si>
   <si>
     <t>Confirmed the existing cart first. The API rejected a second cart. Original cart was not checked again afterward.</t>
@@ -901,14 +838,6 @@
 5. GET /carrinhos?idUsuario=Ujt6HcCXwU3laulg returned 200 OK with quantidade = 0 and carrinhos = []; setup-user response provided the matching user ID, and login/token linkage was checked during review. [E5, E6]</t>
   </si>
   <si>
-    <t>E1. evidence/manual-api/cart/TC-CART-003_STOCK_BEFORE.png
-E2. evidence/manual-api/cart/TC-CART-003_INSUFFICIENT_STOCK_REQUEST.png
-E3. evidence/manual-api/cart/TC-CART-003_INSUFFICIENT_STOCK_RESPONSE.png
-E4. evidence/manual-api/cart/TC-CART-003_STOCK_AFTER.png
-E5. evidence/manual-api/cart/TC-CART-003_VERIFY_NO_CART_RESPONSE.png
-E6. evidence/manual-api/cart/TC-CART-003_USER_SETUP_RESPONSE.png (optional supporting evidence; redact password)</t>
-  </si>
-  <si>
     <t>API rejected the request; stock stayed at 642. No cart was found for the test user. User/token match was checked. Redact secrets.</t>
   </si>
   <si>
@@ -919,13 +848,6 @@
 2. POST /carrinhos returned 400 Bad Request. [E3]
 3. Response message was 'Produto não encontrado'; item identified idProduto = ZZZZ9999XXXX8888, quantidade = 2 and index = 0. [E3]
 4. GET /carrinhos?idUsuario=4NOVKleR5mXplsyX returned 200 OK with quantidade = 0 and carrinhos = []; the user's setup response recorded the corresponding User ID. [E4, E5]</t>
-  </si>
-  <si>
-    <t>E1. evidence/manual-api/cart/TC-CART-004_INVALID_PRODUCT_CHECK.png
-E2. evidence/manual-api/cart/TC-CART-004_INVALID_PRODUCT_REQUEST.png
-E3. evidence/manual-api/cart/TC-CART-004_INVALID_PRODUCT_RESPONSE.png
-E4. evidence/manual-api/cart/TC-CART-004_VERIFY_NO_CART_RESPONSE.png
-E5. evidence/manual-api/cart/TC-CART-004_USER_SETUP_RESPONSE.png (supporting; redact password)</t>
   </si>
   <si>
     <t>API rejected the unknown product ID. No cart was found for the queried user. Original token-to-user match still needs confirmation.</t>
@@ -940,9 +862,9 @@
     <numFmt numFmtId="177" formatCode="_-&quot;฿&quot;* #,##0.00_-;\-&quot;฿&quot;* #,##0.00_-;_-&quot;฿&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="178" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="179" formatCode="_-&quot;฿&quot;* #,##0_-;\-&quot;฿&quot;* #,##0_-;_-&quot;฿&quot;* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="180" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="180" formatCode="dd\ mmm\ yyyy"/>
   </numFmts>
-  <fonts count="33">
+  <fonts count="34">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -962,6 +884,13 @@
       <charset val="134"/>
     </font>
     <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFEAF2FC"/>
+      <name val="Carlito"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color rgb="FFEAF2FC"/>
       <name val="Carlito"/>
@@ -970,18 +899,11 @@
     <font>
       <b/>
       <sz val="10"/>
-      <color rgb="FFEAF2FC"/>
-      <name val="Carlito"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="10"/>
       <color rgb="FF526179"/>
       <name val="Carlito"/>
       <charset val="134"/>
     </font>
     <font>
-      <b/>
       <sz val="10"/>
       <color rgb="FF526179"/>
       <name val="Carlito"/>
@@ -1011,6 +933,23 @@
     <font>
       <b/>
       <sz val="10"/>
+      <name val="Carlito"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Carlito"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1664BC"/>
+      <name val="Carlito"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
       <color rgb="FF182B43"/>
       <name val="Carlito"/>
       <charset val="134"/>
@@ -1018,20 +957,6 @@
     <font>
       <sz val="10"/>
       <color rgb="FF182B43"/>
-      <name val="Carlito"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FF00B050"/>
-      <name val="Carlito"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FFFF0000"/>
       <name val="Carlito"/>
       <charset val="134"/>
     </font>
@@ -1159,7 +1084,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="41">
+  <fills count="43">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1198,19 +1123,31 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF0E756E"/>
+        <fgColor theme="3" tint="0.1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F6FB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4F7FB"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF4F7FB"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1401,7 +1338,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -1437,32 +1374,6 @@
       <bottom style="hair">
         <color auto="1"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="hair">
-        <color auto="1"/>
-      </left>
-      <right style="hair">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="hair">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="hair">
-        <color auto="1"/>
-      </left>
-      <right style="hair">
-        <color auto="1"/>
-      </right>
-      <top style="hair">
-        <color auto="1"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -1566,31 +1477,28 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="178" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="179" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1599,124 +1507,135 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="13" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1730,20 +1649,14 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1755,149 +1668,113 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="180" fontId="11" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="180" fontId="11" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="180" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="180" fontId="11" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="180" fontId="11" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="180" fontId="11" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="180" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1955,7 +1832,7 @@
   <dxfs count="22">
     <dxf>
       <font>
-        <b val="1"/>
+        <color auto="1"/>
       </font>
     </dxf>
     <dxf>
@@ -2224,24 +2101,7 @@
     <tableColumn id="11" name="Test Steps"/>
     <tableColumn id="12" name="Expected HTTP Status"/>
     <tableColumn id="13" name="Expected Response / Behavior"/>
-    <tableColumn id="14" name="Automation Status"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ServeRestTestExecution" displayName="ServeRestTestExecution" ref="A6:I16" totalsRowShown="0">
-  <tableColumns count="9">
-    <tableColumn id="1" name="Run ID"/>
-    <tableColumn id="2" name="Test Case ID"/>
-    <tableColumn id="3" name="Execution Date"/>
-    <tableColumn id="4" name="Environment"/>
-    <tableColumn id="5" name="Actual HTTP Status"/>
-    <tableColumn id="6" name="Actual Response / Result"/>
-    <tableColumn id="7" name="Test Status" dataDxfId="0"/>
-    <tableColumn id="8" name="Evidence"/>
-    <tableColumn id="9" name="Remarks / Defect ID"/>
+    <tableColumn id="14" name="Automation Status" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2449,89 +2309,89 @@
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
     <col min="4" max="4" width="37" customWidth="1"/>
-    <col min="5" max="5" width="15.25" style="2" customWidth="1"/>
-    <col min="6" max="6" width="12" style="2" customWidth="1"/>
+    <col min="5" max="5" width="15.25" style="28" customWidth="1"/>
+    <col min="6" max="6" width="12" style="28" customWidth="1"/>
     <col min="7" max="7" width="42" customWidth="1"/>
-    <col min="8" max="8" width="15" style="2" customWidth="1"/>
+    <col min="8" max="8" width="15" style="28" customWidth="1"/>
     <col min="9" max="9" width="29.875" customWidth="1"/>
     <col min="10" max="10" width="45" customWidth="1"/>
     <col min="11" max="11" width="49" customWidth="1"/>
-    <col min="12" max="12" width="26.375" style="2" customWidth="1"/>
+    <col min="12" max="12" width="26.375" style="28" customWidth="1"/>
     <col min="13" max="13" width="50" customWidth="1"/>
-    <col min="14" max="14" width="21" style="51" customWidth="1"/>
+    <col min="14" max="14" width="21" style="29" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1" spans="1:14">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:14">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="7"/>
-      <c r="M2" s="6"/>
-      <c r="N2" s="7"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="9"/>
+      <c r="N2" s="8"/>
     </row>
     <row r="3" ht="27" customHeight="1" spans="1:14">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="9"/>
-      <c r="L3" s="10"/>
-      <c r="M3" s="9"/>
-      <c r="N3" s="52"/>
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="30"/>
+      <c r="J3" s="30"/>
+      <c r="K3" s="30"/>
+      <c r="L3" s="31"/>
+      <c r="M3" s="30"/>
+      <c r="N3" s="32"/>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:14">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="12"/>
-      <c r="G4" s="12"/>
-      <c r="H4" s="12"/>
-      <c r="I4" s="12"/>
-      <c r="J4" s="12"/>
-      <c r="K4" s="12"/>
-      <c r="L4" s="12"/>
-      <c r="M4" s="12"/>
-      <c r="N4" s="53"/>
+      <c r="B4" s="33"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="33"/>
+      <c r="G4" s="33"/>
+      <c r="H4" s="33"/>
+      <c r="I4" s="33"/>
+      <c r="J4" s="33"/>
+      <c r="K4" s="33"/>
+      <c r="L4" s="33"/>
+      <c r="M4" s="33"/>
+      <c r="N4" s="34"/>
     </row>
     <row r="5" ht="24" customHeight="1" spans="1:14">
       <c r="A5" s="14" t="s">
@@ -2558,912 +2418,912 @@
       <c r="N5" s="14"/>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:14">
-      <c r="A6" s="54" t="s">
+      <c r="A6" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="54" t="s">
+      <c r="B6" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="54" t="s">
+      <c r="C6" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="54" t="s">
+      <c r="D6" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="54" t="s">
+      <c r="E6" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="54" t="s">
+      <c r="F6" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="54" t="s">
+      <c r="G6" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="54" t="s">
+      <c r="H6" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="I6" s="54" t="s">
+      <c r="I6" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="J6" s="54" t="s">
+      <c r="J6" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="K6" s="54" t="s">
+      <c r="K6" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="L6" s="54" t="s">
+      <c r="L6" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="M6" s="54" t="s">
+      <c r="M6" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="N6" s="54" t="s">
+      <c r="N6" s="17" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="7" ht="100" customHeight="1" spans="1:14">
-      <c r="A7" s="23" t="s">
+      <c r="A7" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="23" t="s">
+      <c r="B7" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="C7" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="26" t="s">
+      <c r="D7" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="23" t="s">
+      <c r="E7" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="F7" s="55" t="s">
+      <c r="F7" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="G7" s="26" t="s">
+      <c r="G7" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="H7" s="55" t="s">
+      <c r="H7" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="I7" s="25" t="s">
+      <c r="I7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="J7" s="26" t="s">
+      <c r="J7" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="K7" s="26" t="s">
+      <c r="K7" s="37" t="s">
         <v>32</v>
       </c>
-      <c r="L7" s="23">
+      <c r="L7" s="35">
         <v>201</v>
       </c>
-      <c r="M7" s="26" t="s">
+      <c r="M7" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="N7" s="56" t="s">
+      <c r="N7" s="39" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="8" ht="100" customHeight="1" spans="1:14">
-      <c r="A8" s="28" t="s">
+      <c r="A8" s="40" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="28" t="s">
+      <c r="B8" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="30" t="s">
+      <c r="C8" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="31" t="s">
+      <c r="D8" s="42" t="s">
         <v>36</v>
       </c>
-      <c r="E8" s="28" t="s">
+      <c r="E8" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="F8" s="57" t="s">
+      <c r="F8" s="43" t="s">
         <v>27</v>
       </c>
-      <c r="G8" s="31" t="s">
+      <c r="G8" s="42" t="s">
         <v>38</v>
       </c>
-      <c r="H8" s="57" t="s">
+      <c r="H8" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="I8" s="30" t="s">
+      <c r="I8" s="41" t="s">
         <v>30</v>
       </c>
-      <c r="J8" s="31" t="s">
+      <c r="J8" s="42" t="s">
         <v>39</v>
       </c>
-      <c r="K8" s="31" t="s">
+      <c r="K8" s="42" t="s">
         <v>40</v>
       </c>
-      <c r="L8" s="28">
+      <c r="L8" s="40">
         <v>400</v>
       </c>
-      <c r="M8" s="31" t="s">
+      <c r="M8" s="42" t="s">
         <v>41</v>
       </c>
-      <c r="N8" s="58" t="s">
+      <c r="N8" s="44" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="9" ht="101" customHeight="1" spans="1:14">
-      <c r="A9" s="23" t="s">
+      <c r="A9" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="25" t="s">
+      <c r="C9" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="26" t="s">
+      <c r="D9" s="37" t="s">
         <v>43</v>
       </c>
-      <c r="E9" s="23" t="s">
+      <c r="E9" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="F9" s="55" t="s">
+      <c r="F9" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="G9" s="26" t="s">
+      <c r="G9" s="37" t="s">
         <v>44</v>
       </c>
-      <c r="H9" s="55" t="s">
+      <c r="H9" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="I9" s="25" t="s">
+      <c r="I9" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="J9" s="26" t="s">
+      <c r="J9" s="37" t="s">
         <v>45</v>
       </c>
-      <c r="K9" s="26" t="s">
+      <c r="K9" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="L9" s="23">
+      <c r="L9" s="35">
         <v>400</v>
       </c>
-      <c r="M9" s="26" t="s">
+      <c r="M9" s="37" t="s">
         <v>47</v>
       </c>
-      <c r="N9" s="59" t="s">
+      <c r="N9" s="39" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="10" ht="118" customHeight="1" spans="1:14">
-      <c r="A10" s="28" t="s">
+      <c r="A10" s="40" t="s">
         <v>49</v>
       </c>
-      <c r="B10" s="28" t="s">
+      <c r="B10" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="30" t="s">
+      <c r="C10" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="D10" s="31" t="s">
+      <c r="D10" s="42" t="s">
         <v>50</v>
       </c>
-      <c r="E10" s="28" t="s">
+      <c r="E10" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="F10" s="57" t="s">
+      <c r="F10" s="43" t="s">
         <v>27</v>
       </c>
-      <c r="G10" s="31" t="s">
+      <c r="G10" s="42" t="s">
         <v>51</v>
       </c>
-      <c r="H10" s="57" t="s">
+      <c r="H10" s="43" t="s">
         <v>52</v>
       </c>
-      <c r="I10" s="30" t="s">
+      <c r="I10" s="41" t="s">
         <v>53</v>
       </c>
-      <c r="J10" s="31" t="s">
+      <c r="J10" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="K10" s="31" t="s">
+      <c r="K10" s="42" t="s">
         <v>55</v>
       </c>
-      <c r="L10" s="28">
+      <c r="L10" s="40">
         <v>200</v>
       </c>
-      <c r="M10" s="31" t="s">
+      <c r="M10" s="42" t="s">
         <v>56</v>
       </c>
-      <c r="N10" s="60" t="s">
+      <c r="N10" s="44" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="11" ht="108" customHeight="1" spans="1:14">
-      <c r="A11" s="23" t="s">
+      <c r="A11" s="35" t="s">
         <v>57</v>
       </c>
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="35" t="s">
         <v>58</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="C11" s="36" t="s">
         <v>59</v>
       </c>
-      <c r="D11" s="26" t="s">
+      <c r="D11" s="37" t="s">
         <v>60</v>
       </c>
-      <c r="E11" s="23" t="s">
+      <c r="E11" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="F11" s="55" t="s">
+      <c r="F11" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="G11" s="26" t="s">
+      <c r="G11" s="37" t="s">
         <v>61</v>
       </c>
-      <c r="H11" s="55" t="s">
+      <c r="H11" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="I11" s="25" t="s">
+      <c r="I11" s="36" t="s">
         <v>62</v>
       </c>
-      <c r="J11" s="26" t="s">
+      <c r="J11" s="37" t="s">
         <v>63</v>
       </c>
-      <c r="K11" s="26" t="s">
+      <c r="K11" s="37" t="s">
         <v>64</v>
       </c>
-      <c r="L11" s="23">
+      <c r="L11" s="35">
         <v>200</v>
       </c>
-      <c r="M11" s="26" t="s">
+      <c r="M11" s="37" t="s">
         <v>65</v>
       </c>
-      <c r="N11" s="56" t="s">
+      <c r="N11" s="39" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="12" ht="122" customHeight="1" spans="1:14">
-      <c r="A12" s="28" t="s">
+      <c r="A12" s="40" t="s">
         <v>66</v>
       </c>
-      <c r="B12" s="28" t="s">
+      <c r="B12" s="40" t="s">
         <v>58</v>
       </c>
-      <c r="C12" s="30" t="s">
+      <c r="C12" s="41" t="s">
         <v>59</v>
       </c>
-      <c r="D12" s="31" t="s">
+      <c r="D12" s="42" t="s">
         <v>67</v>
       </c>
-      <c r="E12" s="28" t="s">
+      <c r="E12" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="F12" s="57" t="s">
+      <c r="F12" s="43" t="s">
         <v>27</v>
       </c>
-      <c r="G12" s="31" t="s">
+      <c r="G12" s="42" t="s">
         <v>68</v>
       </c>
-      <c r="H12" s="57" t="s">
+      <c r="H12" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="I12" s="30" t="s">
+      <c r="I12" s="41" t="s">
         <v>62</v>
       </c>
-      <c r="J12" s="31" t="s">
+      <c r="J12" s="42" t="s">
         <v>69</v>
       </c>
-      <c r="K12" s="31" t="s">
+      <c r="K12" s="42" t="s">
         <v>70</v>
       </c>
-      <c r="L12" s="28">
+      <c r="L12" s="40">
         <v>401</v>
       </c>
-      <c r="M12" s="31" t="s">
+      <c r="M12" s="42" t="s">
         <v>71</v>
       </c>
-      <c r="N12" s="58" t="s">
+      <c r="N12" s="44" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="13" ht="137" customHeight="1" spans="1:14">
-      <c r="A13" s="23" t="s">
+      <c r="A13" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="B13" s="23" t="s">
+      <c r="B13" s="35" t="s">
         <v>58</v>
       </c>
-      <c r="C13" s="25" t="s">
+      <c r="C13" s="36" t="s">
         <v>59</v>
       </c>
-      <c r="D13" s="26" t="s">
+      <c r="D13" s="37" t="s">
         <v>73</v>
       </c>
-      <c r="E13" s="23" t="s">
+      <c r="E13" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="F13" s="55" t="s">
+      <c r="F13" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="G13" s="26" t="s">
+      <c r="G13" s="37" t="s">
         <v>74</v>
       </c>
-      <c r="H13" s="55" t="s">
+      <c r="H13" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="I13" s="25" t="s">
+      <c r="I13" s="36" t="s">
         <v>62</v>
       </c>
-      <c r="J13" s="26" t="s">
+      <c r="J13" s="37" t="s">
         <v>75</v>
       </c>
-      <c r="K13" s="26" t="s">
+      <c r="K13" s="37" t="s">
         <v>76</v>
       </c>
-      <c r="L13" s="23">
+      <c r="L13" s="35">
         <v>401</v>
       </c>
-      <c r="M13" s="26" t="s">
+      <c r="M13" s="37" t="s">
         <v>77</v>
       </c>
-      <c r="N13" s="59" t="s">
+      <c r="N13" s="39" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="14" ht="126" customHeight="1" spans="1:14">
-      <c r="A14" s="28" t="s">
+      <c r="A14" s="40" t="s">
         <v>78</v>
       </c>
-      <c r="B14" s="28" t="s">
+      <c r="B14" s="40" t="s">
         <v>58</v>
       </c>
-      <c r="C14" s="30" t="s">
+      <c r="C14" s="41" t="s">
         <v>59</v>
       </c>
-      <c r="D14" s="31" t="s">
+      <c r="D14" s="42" t="s">
         <v>79</v>
       </c>
-      <c r="E14" s="28" t="s">
+      <c r="E14" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="F14" s="57" t="s">
+      <c r="F14" s="43" t="s">
         <v>27</v>
       </c>
-      <c r="G14" s="31" t="s">
+      <c r="G14" s="42" t="s">
         <v>80</v>
       </c>
-      <c r="H14" s="57" t="s">
+      <c r="H14" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="I14" s="30" t="s">
+      <c r="I14" s="41" t="s">
         <v>62</v>
       </c>
-      <c r="J14" s="31" t="s">
+      <c r="J14" s="42" t="s">
         <v>81</v>
       </c>
-      <c r="K14" s="31" t="s">
+      <c r="K14" s="42" t="s">
         <v>82</v>
       </c>
-      <c r="L14" s="28">
+      <c r="L14" s="40">
         <v>400</v>
       </c>
-      <c r="M14" s="31" t="s">
+      <c r="M14" s="42" t="s">
         <v>83</v>
       </c>
-      <c r="N14" s="60" t="s">
+      <c r="N14" s="44" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="15" ht="118" customHeight="1" spans="1:14">
-      <c r="A15" s="23" t="s">
+      <c r="A15" s="35" t="s">
         <v>84</v>
       </c>
-      <c r="B15" s="23" t="s">
+      <c r="B15" s="35" t="s">
         <v>85</v>
       </c>
-      <c r="C15" s="25" t="s">
+      <c r="C15" s="36" t="s">
         <v>86</v>
       </c>
-      <c r="D15" s="26" t="s">
+      <c r="D15" s="37" t="s">
         <v>87</v>
       </c>
-      <c r="E15" s="23" t="s">
+      <c r="E15" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="F15" s="55" t="s">
+      <c r="F15" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="G15" s="26" t="s">
+      <c r="G15" s="37" t="s">
         <v>88</v>
       </c>
-      <c r="H15" s="55" t="s">
+      <c r="H15" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="I15" s="25" t="s">
+      <c r="I15" s="36" t="s">
         <v>89</v>
       </c>
-      <c r="J15" s="26" t="s">
+      <c r="J15" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="K15" s="26" t="s">
+      <c r="K15" s="37" t="s">
         <v>91</v>
       </c>
-      <c r="L15" s="23">
+      <c r="L15" s="35">
         <v>200</v>
       </c>
-      <c r="M15" s="26" t="s">
+      <c r="M15" s="37" t="s">
         <v>92</v>
       </c>
-      <c r="N15" s="59" t="s">
+      <c r="N15" s="39" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="16" ht="144" customHeight="1" spans="1:14">
-      <c r="A16" s="28" t="s">
+      <c r="A16" s="40" t="s">
         <v>93</v>
       </c>
-      <c r="B16" s="28" t="s">
+      <c r="B16" s="40" t="s">
         <v>94</v>
       </c>
-      <c r="C16" s="30" t="s">
+      <c r="C16" s="41" t="s">
         <v>86</v>
       </c>
-      <c r="D16" s="31" t="s">
+      <c r="D16" s="42" t="s">
         <v>95</v>
       </c>
-      <c r="E16" s="28" t="s">
+      <c r="E16" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="F16" s="57" t="s">
+      <c r="F16" s="43" t="s">
         <v>27</v>
       </c>
-      <c r="G16" s="31" t="s">
+      <c r="G16" s="42" t="s">
         <v>96</v>
       </c>
-      <c r="H16" s="57" t="s">
+      <c r="H16" s="43" t="s">
         <v>52</v>
       </c>
-      <c r="I16" s="30" t="s">
+      <c r="I16" s="41" t="s">
         <v>97</v>
       </c>
-      <c r="J16" s="31" t="s">
+      <c r="J16" s="42" t="s">
         <v>98</v>
       </c>
-      <c r="K16" s="31" t="s">
+      <c r="K16" s="42" t="s">
         <v>99</v>
       </c>
-      <c r="L16" s="28">
+      <c r="L16" s="40">
         <v>200</v>
       </c>
-      <c r="M16" s="31" t="s">
+      <c r="M16" s="42" t="s">
         <v>100</v>
       </c>
-      <c r="N16" s="60" t="s">
+      <c r="N16" s="44" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="17" ht="120" customHeight="1" spans="1:14">
-      <c r="A17" s="23" t="s">
+      <c r="A17" s="35" t="s">
         <v>101</v>
       </c>
-      <c r="B17" s="23" t="s">
+      <c r="B17" s="35" t="s">
         <v>102</v>
       </c>
-      <c r="C17" s="25" t="s">
+      <c r="C17" s="36" t="s">
         <v>86</v>
       </c>
-      <c r="D17" s="26" t="s">
+      <c r="D17" s="37" t="s">
         <v>103</v>
       </c>
-      <c r="E17" s="23" t="s">
+      <c r="E17" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="F17" s="55" t="s">
+      <c r="F17" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="G17" s="26" t="s">
+      <c r="G17" s="37" t="s">
         <v>104</v>
       </c>
-      <c r="H17" s="55" t="s">
+      <c r="H17" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="I17" s="25" t="s">
+      <c r="I17" s="36" t="s">
         <v>89</v>
       </c>
-      <c r="J17" s="26" t="s">
+      <c r="J17" s="37" t="s">
         <v>105</v>
       </c>
-      <c r="K17" s="26" t="s">
+      <c r="K17" s="37" t="s">
         <v>106</v>
       </c>
-      <c r="L17" s="23">
+      <c r="L17" s="35">
         <v>201</v>
       </c>
-      <c r="M17" s="26" t="s">
+      <c r="M17" s="37" t="s">
         <v>107</v>
       </c>
-      <c r="N17" s="56" t="s">
+      <c r="N17" s="39" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="18" ht="182" customHeight="1" spans="1:14">
-      <c r="A18" s="28" t="s">
+      <c r="A18" s="40" t="s">
         <v>108</v>
       </c>
-      <c r="B18" s="61" t="s">
+      <c r="B18" s="45" t="s">
         <v>109</v>
       </c>
-      <c r="C18" s="62" t="s">
+      <c r="C18" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="D18" s="31" t="s">
+      <c r="D18" s="42" t="s">
         <v>110</v>
       </c>
-      <c r="E18" s="28" t="s">
+      <c r="E18" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="F18" s="57" t="s">
+      <c r="F18" s="43" t="s">
         <v>27</v>
       </c>
-      <c r="G18" s="31" t="s">
+      <c r="G18" s="42" t="s">
         <v>111</v>
       </c>
-      <c r="H18" s="57" t="s">
+      <c r="H18" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="I18" s="30" t="s">
+      <c r="I18" s="41" t="s">
         <v>89</v>
       </c>
-      <c r="J18" s="31" t="s">
+      <c r="J18" s="42" t="s">
         <v>112</v>
       </c>
-      <c r="K18" s="31" t="s">
+      <c r="K18" s="42" t="s">
         <v>113</v>
       </c>
-      <c r="L18" s="28">
+      <c r="L18" s="40">
         <v>400</v>
       </c>
-      <c r="M18" s="32" t="s">
+      <c r="M18" s="47" t="s">
         <v>114</v>
       </c>
-      <c r="N18" s="63" t="s">
+      <c r="N18" s="48" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="19" ht="200" customHeight="1" spans="1:14">
-      <c r="A19" s="23" t="s">
+      <c r="A19" s="35" t="s">
         <v>115</v>
       </c>
-      <c r="B19" s="23" t="s">
+      <c r="B19" s="35" t="s">
         <v>116</v>
       </c>
-      <c r="C19" s="25" t="s">
+      <c r="C19" s="36" t="s">
         <v>117</v>
       </c>
-      <c r="D19" s="27" t="s">
+      <c r="D19" s="49" t="s">
         <v>118</v>
       </c>
-      <c r="E19" s="23" t="s">
+      <c r="E19" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="F19" s="55" t="s">
+      <c r="F19" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="G19" s="26" t="s">
+      <c r="G19" s="37" t="s">
         <v>119</v>
       </c>
-      <c r="H19" s="55" t="s">
+      <c r="H19" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="I19" s="25" t="s">
+      <c r="I19" s="36" t="s">
         <v>120</v>
       </c>
-      <c r="J19" s="26" t="s">
+      <c r="J19" s="37" t="s">
         <v>121</v>
       </c>
-      <c r="K19" s="26" t="s">
+      <c r="K19" s="37" t="s">
         <v>122</v>
       </c>
-      <c r="L19" s="23">
+      <c r="L19" s="35">
         <v>201</v>
       </c>
-      <c r="M19" s="26" t="s">
+      <c r="M19" s="37" t="s">
         <v>123</v>
       </c>
-      <c r="N19" s="56" t="s">
+      <c r="N19" s="39" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="20" ht="200" customHeight="1" spans="1:14">
-      <c r="A20" s="28" t="s">
+      <c r="A20" s="40" t="s">
         <v>124</v>
       </c>
-      <c r="B20" s="28" t="s">
+      <c r="B20" s="40" t="s">
         <v>125</v>
       </c>
-      <c r="C20" s="30" t="s">
+      <c r="C20" s="41" t="s">
         <v>117</v>
       </c>
-      <c r="D20" s="31" t="s">
+      <c r="D20" s="42" t="s">
         <v>126</v>
       </c>
-      <c r="E20" s="28" t="s">
+      <c r="E20" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="F20" s="57" t="s">
+      <c r="F20" s="43" t="s">
         <v>27</v>
       </c>
-      <c r="G20" s="31" t="s">
+      <c r="G20" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="H20" s="57" t="s">
+      <c r="H20" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="I20" s="30" t="s">
+      <c r="I20" s="41" t="s">
         <v>120</v>
       </c>
-      <c r="J20" s="31" t="s">
+      <c r="J20" s="42" t="s">
         <v>128</v>
       </c>
-      <c r="K20" s="31" t="s">
+      <c r="K20" s="42" t="s">
         <v>129</v>
       </c>
-      <c r="L20" s="28">
+      <c r="L20" s="40">
         <v>400</v>
       </c>
-      <c r="M20" s="31" t="s">
+      <c r="M20" s="42" t="s">
         <v>130</v>
       </c>
-      <c r="N20" s="60" t="s">
+      <c r="N20" s="44" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="21" ht="218" customHeight="1" spans="1:14">
-      <c r="A21" s="23" t="s">
+      <c r="A21" s="35" t="s">
         <v>131</v>
       </c>
-      <c r="B21" s="23" t="s">
+      <c r="B21" s="35" t="s">
         <v>132</v>
       </c>
-      <c r="C21" s="25" t="s">
+      <c r="C21" s="36" t="s">
         <v>117</v>
       </c>
-      <c r="D21" s="26" t="s">
+      <c r="D21" s="37" t="s">
         <v>133</v>
       </c>
-      <c r="E21" s="23" t="s">
+      <c r="E21" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="F21" s="55" t="s">
+      <c r="F21" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="G21" s="26" t="s">
+      <c r="G21" s="37" t="s">
         <v>134</v>
       </c>
-      <c r="H21" s="55" t="s">
+      <c r="H21" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="I21" s="25" t="s">
+      <c r="I21" s="36" t="s">
         <v>120</v>
       </c>
-      <c r="J21" s="26" t="s">
+      <c r="J21" s="37" t="s">
         <v>135</v>
       </c>
-      <c r="K21" s="26" t="s">
+      <c r="K21" s="37" t="s">
         <v>136</v>
       </c>
-      <c r="L21" s="23">
+      <c r="L21" s="35">
         <v>400</v>
       </c>
-      <c r="M21" s="26" t="s">
+      <c r="M21" s="37" t="s">
         <v>137</v>
       </c>
-      <c r="N21" s="56" t="s">
+      <c r="N21" s="39" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="22" ht="200" customHeight="1" spans="1:14">
-      <c r="A22" s="28" t="s">
+      <c r="A22" s="40" t="s">
         <v>138</v>
       </c>
-      <c r="B22" s="28" t="s">
+      <c r="B22" s="40" t="s">
         <v>139</v>
       </c>
-      <c r="C22" s="30" t="s">
+      <c r="C22" s="41" t="s">
         <v>117</v>
       </c>
-      <c r="D22" s="30" t="s">
+      <c r="D22" s="41" t="s">
         <v>140</v>
       </c>
-      <c r="E22" s="28" t="s">
+      <c r="E22" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="F22" s="57" t="s">
+      <c r="F22" s="43" t="s">
         <v>27</v>
       </c>
-      <c r="G22" s="31" t="s">
+      <c r="G22" s="42" t="s">
         <v>141</v>
       </c>
-      <c r="H22" s="57" t="s">
+      <c r="H22" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="I22" s="30" t="s">
+      <c r="I22" s="41" t="s">
         <v>120</v>
       </c>
-      <c r="J22" s="31" t="s">
+      <c r="J22" s="42" t="s">
         <v>142</v>
       </c>
-      <c r="K22" s="31" t="s">
+      <c r="K22" s="42" t="s">
         <v>143</v>
       </c>
-      <c r="L22" s="28">
+      <c r="L22" s="40">
         <v>400</v>
       </c>
-      <c r="M22" s="31" t="s">
+      <c r="M22" s="42" t="s">
         <v>144</v>
       </c>
-      <c r="N22" s="60" t="s">
+      <c r="N22" s="44" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="23" ht="88" customHeight="1" spans="1:14">
-      <c r="A23" s="38"/>
-      <c r="B23" s="38"/>
-      <c r="C23" s="40"/>
-      <c r="D23" s="40"/>
-      <c r="E23" s="38"/>
-      <c r="F23" s="64"/>
-      <c r="G23" s="40"/>
-      <c r="H23" s="64"/>
-      <c r="I23" s="40"/>
-      <c r="J23" s="40"/>
-      <c r="K23" s="40"/>
-      <c r="L23" s="38"/>
-      <c r="M23" s="40"/>
-      <c r="N23" s="65"/>
+      <c r="A23" s="50"/>
+      <c r="B23" s="50"/>
+      <c r="C23" s="51"/>
+      <c r="D23" s="51"/>
+      <c r="E23" s="50"/>
+      <c r="F23" s="52"/>
+      <c r="G23" s="51"/>
+      <c r="H23" s="52"/>
+      <c r="I23" s="51"/>
+      <c r="J23" s="51"/>
+      <c r="K23" s="51"/>
+      <c r="L23" s="50"/>
+      <c r="M23" s="51"/>
+      <c r="N23" s="53"/>
     </row>
     <row r="24" ht="58" customHeight="1" spans="1:14">
-      <c r="A24" s="38"/>
-      <c r="B24" s="38"/>
-      <c r="C24" s="40"/>
-      <c r="D24" s="40"/>
-      <c r="E24" s="38"/>
-      <c r="F24" s="64"/>
-      <c r="G24" s="40"/>
-      <c r="H24" s="64"/>
-      <c r="I24" s="40"/>
-      <c r="J24" s="40"/>
-      <c r="K24" s="40"/>
-      <c r="L24" s="38"/>
-      <c r="M24" s="40"/>
-      <c r="N24" s="65"/>
+      <c r="A24" s="50"/>
+      <c r="B24" s="50"/>
+      <c r="C24" s="51"/>
+      <c r="D24" s="51"/>
+      <c r="E24" s="50"/>
+      <c r="F24" s="52"/>
+      <c r="G24" s="51"/>
+      <c r="H24" s="52"/>
+      <c r="I24" s="51"/>
+      <c r="J24" s="51"/>
+      <c r="K24" s="51"/>
+      <c r="L24" s="50"/>
+      <c r="M24" s="51"/>
+      <c r="N24" s="53"/>
     </row>
     <row r="25" ht="58" customHeight="1" spans="1:14">
-      <c r="A25" s="38"/>
-      <c r="B25" s="38"/>
-      <c r="C25" s="40"/>
-      <c r="D25" s="40"/>
-      <c r="E25" s="38"/>
-      <c r="F25" s="64"/>
-      <c r="G25" s="40"/>
-      <c r="H25" s="64"/>
-      <c r="I25" s="40"/>
-      <c r="J25" s="40"/>
-      <c r="K25" s="40"/>
-      <c r="L25" s="38"/>
-      <c r="M25" s="40"/>
-      <c r="N25" s="65"/>
+      <c r="A25" s="50"/>
+      <c r="B25" s="50"/>
+      <c r="C25" s="51"/>
+      <c r="D25" s="51"/>
+      <c r="E25" s="50"/>
+      <c r="F25" s="52"/>
+      <c r="G25" s="51"/>
+      <c r="H25" s="52"/>
+      <c r="I25" s="51"/>
+      <c r="J25" s="51"/>
+      <c r="K25" s="51"/>
+      <c r="L25" s="50"/>
+      <c r="M25" s="51"/>
+      <c r="N25" s="53"/>
     </row>
     <row r="26" ht="58" customHeight="1" spans="1:14">
-      <c r="A26" s="38"/>
-      <c r="B26" s="38"/>
-      <c r="C26" s="40"/>
-      <c r="D26" s="40"/>
-      <c r="E26" s="38"/>
-      <c r="F26" s="64"/>
-      <c r="G26" s="40"/>
-      <c r="H26" s="64"/>
-      <c r="I26" s="40"/>
-      <c r="J26" s="40"/>
-      <c r="K26" s="40"/>
-      <c r="L26" s="38"/>
-      <c r="M26" s="40"/>
-      <c r="N26" s="65"/>
+      <c r="A26" s="50"/>
+      <c r="B26" s="50"/>
+      <c r="C26" s="51"/>
+      <c r="D26" s="51"/>
+      <c r="E26" s="50"/>
+      <c r="F26" s="52"/>
+      <c r="G26" s="51"/>
+      <c r="H26" s="52"/>
+      <c r="I26" s="51"/>
+      <c r="J26" s="51"/>
+      <c r="K26" s="51"/>
+      <c r="L26" s="50"/>
+      <c r="M26" s="51"/>
+      <c r="N26" s="53"/>
     </row>
     <row r="27" ht="58" customHeight="1" spans="1:14">
-      <c r="A27" s="38"/>
-      <c r="B27" s="38"/>
-      <c r="C27" s="40"/>
-      <c r="D27" s="40"/>
-      <c r="E27" s="38"/>
-      <c r="F27" s="64"/>
-      <c r="G27" s="40"/>
-      <c r="H27" s="64"/>
-      <c r="I27" s="40"/>
-      <c r="J27" s="40"/>
-      <c r="K27" s="40"/>
-      <c r="L27" s="38"/>
-      <c r="M27" s="40"/>
-      <c r="N27" s="65"/>
+      <c r="A27" s="50"/>
+      <c r="B27" s="50"/>
+      <c r="C27" s="51"/>
+      <c r="D27" s="51"/>
+      <c r="E27" s="50"/>
+      <c r="F27" s="52"/>
+      <c r="G27" s="51"/>
+      <c r="H27" s="52"/>
+      <c r="I27" s="51"/>
+      <c r="J27" s="51"/>
+      <c r="K27" s="51"/>
+      <c r="L27" s="50"/>
+      <c r="M27" s="51"/>
+      <c r="N27" s="53"/>
     </row>
     <row r="28" ht="58" customHeight="1" spans="1:14">
-      <c r="A28" s="38"/>
-      <c r="B28" s="38"/>
-      <c r="C28" s="40"/>
-      <c r="D28" s="40"/>
-      <c r="E28" s="38"/>
-      <c r="F28" s="64"/>
-      <c r="G28" s="40"/>
-      <c r="H28" s="64"/>
-      <c r="I28" s="40"/>
-      <c r="J28" s="40"/>
-      <c r="K28" s="40"/>
-      <c r="L28" s="38"/>
-      <c r="M28" s="40"/>
-      <c r="N28" s="65"/>
+      <c r="A28" s="50"/>
+      <c r="B28" s="50"/>
+      <c r="C28" s="51"/>
+      <c r="D28" s="51"/>
+      <c r="E28" s="50"/>
+      <c r="F28" s="52"/>
+      <c r="G28" s="51"/>
+      <c r="H28" s="52"/>
+      <c r="I28" s="51"/>
+      <c r="J28" s="51"/>
+      <c r="K28" s="51"/>
+      <c r="L28" s="50"/>
+      <c r="M28" s="51"/>
+      <c r="N28" s="53"/>
     </row>
     <row r="29" ht="58" customHeight="1" spans="1:14">
-      <c r="A29" s="38"/>
-      <c r="B29" s="38"/>
-      <c r="C29" s="40"/>
-      <c r="D29" s="40"/>
-      <c r="E29" s="38"/>
-      <c r="F29" s="64"/>
-      <c r="G29" s="40"/>
-      <c r="H29" s="64"/>
-      <c r="I29" s="40"/>
-      <c r="J29" s="40"/>
-      <c r="K29" s="40"/>
-      <c r="L29" s="38"/>
-      <c r="M29" s="40"/>
-      <c r="N29" s="65"/>
+      <c r="A29" s="50"/>
+      <c r="B29" s="50"/>
+      <c r="C29" s="51"/>
+      <c r="D29" s="51"/>
+      <c r="E29" s="50"/>
+      <c r="F29" s="52"/>
+      <c r="G29" s="51"/>
+      <c r="H29" s="52"/>
+      <c r="I29" s="51"/>
+      <c r="J29" s="51"/>
+      <c r="K29" s="51"/>
+      <c r="L29" s="50"/>
+      <c r="M29" s="51"/>
+      <c r="N29" s="53"/>
     </row>
     <row r="30" ht="58" customHeight="1" spans="1:14">
-      <c r="A30" s="38"/>
-      <c r="B30" s="38"/>
-      <c r="C30" s="40"/>
-      <c r="D30" s="40"/>
-      <c r="E30" s="38"/>
-      <c r="F30" s="64"/>
-      <c r="G30" s="40"/>
-      <c r="H30" s="64"/>
-      <c r="I30" s="40"/>
-      <c r="J30" s="40"/>
-      <c r="K30" s="40"/>
-      <c r="L30" s="38"/>
-      <c r="M30" s="40"/>
-      <c r="N30" s="65"/>
+      <c r="A30" s="50"/>
+      <c r="B30" s="50"/>
+      <c r="C30" s="51"/>
+      <c r="D30" s="51"/>
+      <c r="E30" s="50"/>
+      <c r="F30" s="52"/>
+      <c r="G30" s="51"/>
+      <c r="H30" s="52"/>
+      <c r="I30" s="51"/>
+      <c r="J30" s="51"/>
+      <c r="K30" s="51"/>
+      <c r="L30" s="50"/>
+      <c r="M30" s="51"/>
+      <c r="N30" s="53"/>
     </row>
     <row r="31" ht="58" customHeight="1" spans="1:14">
-      <c r="A31" s="38"/>
-      <c r="B31" s="38"/>
-      <c r="C31" s="40"/>
-      <c r="D31" s="40"/>
-      <c r="E31" s="38"/>
-      <c r="F31" s="64"/>
-      <c r="G31" s="40"/>
-      <c r="H31" s="64"/>
-      <c r="I31" s="40"/>
-      <c r="J31" s="40"/>
-      <c r="K31" s="40"/>
-      <c r="L31" s="38"/>
-      <c r="M31" s="40"/>
-      <c r="N31" s="65"/>
+      <c r="A31" s="50"/>
+      <c r="B31" s="50"/>
+      <c r="C31" s="51"/>
+      <c r="D31" s="51"/>
+      <c r="E31" s="50"/>
+      <c r="F31" s="52"/>
+      <c r="G31" s="51"/>
+      <c r="H31" s="52"/>
+      <c r="I31" s="51"/>
+      <c r="J31" s="51"/>
+      <c r="K31" s="51"/>
+      <c r="L31" s="50"/>
+      <c r="M31" s="51"/>
+      <c r="N31" s="53"/>
     </row>
     <row r="32" ht="58" customHeight="1" spans="1:14">
-      <c r="A32" s="38"/>
-      <c r="B32" s="38"/>
-      <c r="C32" s="40"/>
-      <c r="D32" s="40"/>
-      <c r="E32" s="38"/>
-      <c r="F32" s="64"/>
-      <c r="G32" s="40"/>
-      <c r="H32" s="64"/>
-      <c r="I32" s="40"/>
-      <c r="J32" s="40"/>
-      <c r="K32" s="40"/>
-      <c r="L32" s="38"/>
-      <c r="M32" s="40"/>
-      <c r="N32" s="65"/>
+      <c r="A32" s="50"/>
+      <c r="B32" s="50"/>
+      <c r="C32" s="51"/>
+      <c r="D32" s="51"/>
+      <c r="E32" s="50"/>
+      <c r="F32" s="52"/>
+      <c r="G32" s="51"/>
+      <c r="H32" s="52"/>
+      <c r="I32" s="51"/>
+      <c r="J32" s="51"/>
+      <c r="K32" s="51"/>
+      <c r="L32" s="50"/>
+      <c r="M32" s="51"/>
+      <c r="N32" s="53"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -3493,7 +3353,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="N7:N8 N11:N12 N17:N19 N21" listDataValidation="1"/>
+    <ignoredError sqref="N7:N8 N11:N12 N17:N19" listDataValidation="1"/>
   </ignoredErrors>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -3504,73 +3364,73 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:XFD51"/>
+  <dimension ref="A1:XFD54"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="4" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="19" style="2" customWidth="1"/>
-    <col min="6" max="6" width="89.75" customWidth="1"/>
-    <col min="7" max="7" width="13.75" customWidth="1"/>
-    <col min="8" max="8" width="84.625" style="3" customWidth="1"/>
-    <col min="9" max="9" width="49" customWidth="1"/>
+    <col min="1" max="1" width="13" style="3" customWidth="1"/>
+    <col min="2" max="3" width="18" style="4" customWidth="1"/>
+    <col min="4" max="4" width="20" style="4" customWidth="1"/>
+    <col min="5" max="5" width="17.125" style="3" customWidth="1"/>
+    <col min="6" max="6" width="82.875" customWidth="1"/>
+    <col min="7" max="7" width="12" style="5" customWidth="1"/>
+    <col min="8" max="8" width="72.875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="74.25" customWidth="1"/>
+    <col min="10" max="15" width="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1" spans="1:1024 1025:16384">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="4"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="6"/>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:1024 1025:16384">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="6"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="9"/>
     </row>
-    <row r="3" ht="27" customHeight="1" spans="1:1024 1025:16384">
-      <c r="A3" s="9" t="s">
+    <row r="3" s="1" customFormat="1" ht="27" customHeight="1" spans="1:1024 1025:16384">
+      <c r="A3" s="11" t="s">
         <v>147</v>
       </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="9"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:1024 1025:16384">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="13" t="s">
         <v>148</v>
       </c>
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="12"/>
-      <c r="G4" s="12"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13"/>
       <c r="H4" s="13"/>
-      <c r="I4" s="12"/>
+      <c r="I4" s="13"/>
     </row>
-    <row r="5" s="1" customFormat="1" ht="24" customHeight="1" spans="1:1024 1025:16384">
+    <row r="5" s="2" customFormat="1" ht="24" customHeight="1" spans="1:1024 1025:16384">
       <c r="A5" s="14" t="s">
         <v>149</v>
       </c>
@@ -3586,12 +3446,12 @@
         <v>151</v>
       </c>
       <c r="I5" s="14"/>
-      <c r="J5" s="16"/>
-      <c r="K5" s="16"/>
-      <c r="L5" s="16"/>
-      <c r="M5" s="16"/>
-      <c r="N5" s="16"/>
-      <c r="O5" s="16"/>
+      <c r="J5"/>
+      <c r="K5"/>
+      <c r="L5"/>
+      <c r="M5"/>
+      <c r="N5"/>
+      <c r="O5"/>
       <c r="P5" s="16"/>
       <c r="Q5" s="16"/>
       <c r="R5" s="16"/>
@@ -19991,17 +19851,17 @@
         <v>159</v>
       </c>
     </row>
-    <row r="7" ht="86" customHeight="1" spans="1:1024 1025:16384">
+    <row r="7" ht="34" customHeight="1" spans="1:1024 1025:16384">
       <c r="A7" s="18" t="s">
         <v>160</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="19">
+      <c r="C7" s="20">
         <v>46313</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="D7" s="19" t="s">
         <v>161</v>
       </c>
       <c r="E7" s="18">
@@ -20013,609 +19873,914 @@
       <c r="G7" s="18" t="s">
         <v>163</v>
       </c>
-      <c r="H7" s="22" t="s">
+      <c r="H7" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/user-management/TC-USER-001_CREATE_USER_REQUEST.png","E1 — TC-USER-001_CREATE_USER_REQUEST.png")</f>
+        <v>E1 — TC-USER-001_CREATE_USER_REQUEST.png</v>
+      </c>
+      <c r="I7" s="21" t="s">
         <v>164</v>
       </c>
-      <c r="I7" s="21" t="s">
+    </row>
+    <row r="8" ht="34" customHeight="1" spans="1:1024 1025:16384">
+      <c r="A8" s="18"/>
+      <c r="B8" s="19"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="21"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/user-management/TC-USER-001_CREATE_USER_RESPONSE.png","E2 — TC-USER-001_CREATE_USER_RESPONSE.png")</f>
+        <v>E2 — TC-USER-001_CREATE_USER_RESPONSE.png</v>
+      </c>
+      <c r="I8" s="21"/>
+    </row>
+    <row r="9" ht="34" customHeight="1" spans="1:1024 1025:16384">
+      <c r="A9" s="23" t="s">
         <v>165</v>
       </c>
+      <c r="B9" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" s="25">
+        <v>46313</v>
+      </c>
+      <c r="D9" s="24" t="s">
+        <v>161</v>
+      </c>
+      <c r="E9" s="23">
+        <v>400</v>
+      </c>
+      <c r="F9" s="26" t="s">
+        <v>166</v>
+      </c>
+      <c r="G9" s="23" t="s">
+        <v>163</v>
+      </c>
+      <c r="H9" s="27" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/user-management/TC-USER-002_DUPLICATE_EMAIL_REQUEST.png","E1 — TC-USER-002_DUPLICATE_EMAIL_REQUEST.png")</f>
+        <v>E1 — TC-USER-002_DUPLICATE_EMAIL_REQUEST.png</v>
+      </c>
+      <c r="I9" s="26" t="s">
+        <v>167</v>
+      </c>
     </row>
-    <row r="8" ht="86" customHeight="1" spans="1:1024 1025:16384">
-      <c r="A8" s="23" t="s">
-        <v>166</v>
-      </c>
-      <c r="B8" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="C8" s="24">
+    <row r="10" ht="34" customHeight="1" spans="1:1024 1025:16384">
+      <c r="A10" s="23"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="26"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="27" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/user-management/TC-USER-002_DUPLICATE_EMAIL_RESPONSE.png","E2 — TC-USER-002_DUPLICATE_EMAIL_RESPONSE.png")</f>
+        <v>E2 — TC-USER-002_DUPLICATE_EMAIL_RESPONSE.png</v>
+      </c>
+      <c r="I10" s="26"/>
+    </row>
+    <row r="11" ht="34" customHeight="1" spans="1:1024 1025:16384">
+      <c r="A11" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="B11" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="20">
         <v>46313</v>
       </c>
-      <c r="D8" s="25" t="s">
+      <c r="D11" s="19" t="s">
         <v>161</v>
       </c>
-      <c r="E8" s="23">
+      <c r="E11" s="18">
         <v>400</v>
       </c>
-      <c r="F8" s="26" t="s">
-        <v>167</v>
-      </c>
-      <c r="G8" s="23" t="s">
-        <v>163</v>
-      </c>
-      <c r="H8" s="27" t="s">
-        <v>168</v>
-      </c>
-      <c r="I8" s="26" t="s">
+      <c r="F11" s="21" t="s">
         <v>169</v>
-      </c>
-    </row>
-    <row r="9" ht="86" customHeight="1" spans="1:1024 1025:16384">
-      <c r="A9" s="18" t="s">
-        <v>170</v>
-      </c>
-      <c r="B9" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="C9" s="19">
-        <v>46313</v>
-      </c>
-      <c r="D9" s="20" t="s">
-        <v>161</v>
-      </c>
-      <c r="E9" s="18">
-        <v>400</v>
-      </c>
-      <c r="F9" s="21" t="s">
-        <v>171</v>
-      </c>
-      <c r="G9" s="18" t="s">
-        <v>163</v>
-      </c>
-      <c r="H9" s="22" t="s">
-        <v>172</v>
-      </c>
-      <c r="I9" s="21" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="10" ht="106" customHeight="1" spans="1:1024 1025:16384">
-      <c r="A10" s="23" t="s">
-        <v>174</v>
-      </c>
-      <c r="B10" s="23" t="s">
-        <v>49</v>
-      </c>
-      <c r="C10" s="24">
-        <v>46313</v>
-      </c>
-      <c r="D10" s="25" t="s">
-        <v>161</v>
-      </c>
-      <c r="E10" s="23">
-        <v>200</v>
-      </c>
-      <c r="F10" s="26" t="s">
-        <v>175</v>
-      </c>
-      <c r="G10" s="23" t="s">
-        <v>163</v>
-      </c>
-      <c r="H10" s="27" t="s">
-        <v>176</v>
-      </c>
-      <c r="I10" s="26" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="11" ht="106" customHeight="1" spans="1:1024 1025:16384">
-      <c r="A11" s="18" t="s">
-        <v>178</v>
-      </c>
-      <c r="B11" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="C11" s="19">
-        <v>46313</v>
-      </c>
-      <c r="D11" s="20" t="s">
-        <v>161</v>
-      </c>
-      <c r="E11" s="18">
-        <v>200</v>
-      </c>
-      <c r="F11" s="21" t="s">
-        <v>179</v>
       </c>
       <c r="G11" s="18" t="s">
         <v>163</v>
       </c>
-      <c r="H11" s="22" t="s">
-        <v>180</v>
+      <c r="H11" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/user-management/TC-USER-003_MISSING_EMAIL_REQUEST.png","E1 — TC-USER-003_MISSING_EMAIL_REQUEST.png")</f>
+        <v>E1 — TC-USER-003_MISSING_EMAIL_REQUEST.png</v>
       </c>
       <c r="I11" s="21" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
     </row>
-    <row r="12" ht="107" customHeight="1" spans="1:1024 1025:16384">
-      <c r="A12" s="23" t="s">
-        <v>182</v>
-      </c>
-      <c r="B12" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="C12" s="24">
-        <v>46314</v>
-      </c>
-      <c r="D12" s="25" t="s">
+    <row r="12" ht="34" customHeight="1" spans="1:1024 1025:16384">
+      <c r="A12" s="18"/>
+      <c r="B12" s="19"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/user-management/TC-USER-003_MISSING_EMAIL_RESPONSE.png","E2 — TC-USER-003_MISSING_EMAIL_RESPONSE.png")</f>
+        <v>E2 — TC-USER-003_MISSING_EMAIL_RESPONSE.png</v>
+      </c>
+      <c r="I12" s="21"/>
+    </row>
+    <row r="13" ht="34" customHeight="1" spans="1:1024 1025:16384">
+      <c r="A13" s="23" t="s">
+        <v>171</v>
+      </c>
+      <c r="B13" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="25">
+        <v>46313</v>
+      </c>
+      <c r="D13" s="24" t="s">
         <v>161</v>
       </c>
-      <c r="E12" s="23">
-        <v>401</v>
-      </c>
-      <c r="F12" s="26" t="s">
-        <v>183</v>
-      </c>
-      <c r="G12" s="23" t="s">
+      <c r="E13" s="23">
+        <v>200</v>
+      </c>
+      <c r="F13" s="26" t="s">
+        <v>172</v>
+      </c>
+      <c r="G13" s="23" t="s">
         <v>163</v>
       </c>
-      <c r="H12" s="27" t="s">
-        <v>184</v>
-      </c>
-      <c r="I12" s="26" t="s">
-        <v>185</v>
+      <c r="H13" s="27" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/user-management/TC-USER-004_GET_USER_REQUEST.png","E1 — TC-USER-004_GET_USER_REQUEST.png")</f>
+        <v>E1 — TC-USER-004_GET_USER_REQUEST.png</v>
+      </c>
+      <c r="I13" s="26" t="s">
+        <v>173</v>
       </c>
     </row>
-    <row r="13" ht="111" customHeight="1" spans="1:1024 1025:16384">
-      <c r="A13" s="18" t="s">
-        <v>186</v>
-      </c>
-      <c r="B13" s="18" t="s">
-        <v>72</v>
-      </c>
-      <c r="C13" s="19">
-        <v>46314</v>
-      </c>
-      <c r="D13" s="20" t="s">
-        <v>161</v>
-      </c>
-      <c r="E13" s="18">
-        <v>401</v>
-      </c>
-      <c r="F13" s="21" t="s">
-        <v>187</v>
-      </c>
-      <c r="G13" s="18" t="s">
-        <v>163</v>
-      </c>
-      <c r="H13" s="22" t="s">
-        <v>188</v>
-      </c>
-      <c r="I13" s="21" t="s">
-        <v>189</v>
-      </c>
+    <row r="14" ht="34" customHeight="1" spans="1:1024 1025:16384">
+      <c r="A14" s="23"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="25"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="26"/>
+      <c r="G14" s="23"/>
+      <c r="H14" s="27" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/user-management/TC-USER-004_GET_USER_RESPONSE.png","E2 — TC-USER-004_GET_USER_RESPONSE.png")</f>
+        <v>E2 — TC-USER-004_GET_USER_RESPONSE.png</v>
+      </c>
+      <c r="I14" s="26"/>
     </row>
-    <row r="14" ht="111" customHeight="1" spans="1:1024 1025:16384">
-      <c r="A14" s="23" t="s">
-        <v>190</v>
-      </c>
-      <c r="B14" s="23" t="s">
-        <v>78</v>
-      </c>
-      <c r="C14" s="24">
-        <v>46315</v>
-      </c>
-      <c r="D14" s="25" t="s">
-        <v>161</v>
-      </c>
-      <c r="E14" s="23">
-        <v>400</v>
-      </c>
-      <c r="F14" s="26" t="s">
-        <v>191</v>
-      </c>
-      <c r="G14" s="23" t="s">
-        <v>163</v>
-      </c>
-      <c r="H14" s="27" t="s">
-        <v>192</v>
-      </c>
-      <c r="I14" s="26" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="15" ht="105" customHeight="1" spans="1:1024 1025:16384">
+    <row r="15" ht="34" customHeight="1" spans="1:1024 1025:16384">
       <c r="A15" s="18" t="s">
-        <v>194</v>
-      </c>
-      <c r="B15" s="18" t="s">
-        <v>84</v>
-      </c>
-      <c r="C15" s="19">
-        <v>46315</v>
-      </c>
-      <c r="D15" s="20" t="s">
+        <v>174</v>
+      </c>
+      <c r="B15" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="C15" s="20">
+        <v>46313</v>
+      </c>
+      <c r="D15" s="19" t="s">
         <v>161</v>
       </c>
       <c r="E15" s="18">
         <v>200</v>
       </c>
       <c r="F15" s="21" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
       <c r="G15" s="18" t="s">
         <v>163</v>
       </c>
-      <c r="H15" s="22" t="s">
+      <c r="H15" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/authentication/TC-AUTH-001_VALID_LOGIN_REQUEST.png","E1 — TC-AUTH-001_VALID_LOGIN_REQUEST.png")</f>
+        <v>E1 — TC-AUTH-001_VALID_LOGIN_REQUEST.png</v>
+      </c>
+      <c r="I15" s="21" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1" spans="1:1024 1025:16384">
+      <c r="A16" s="18"/>
+      <c r="B16" s="19"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="18"/>
+      <c r="F16" s="21"/>
+      <c r="G16" s="18"/>
+      <c r="H16" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/authentication/TC-AUTH-001_VALID_LOGIN_RESPONSE.png","E2 — TC-AUTH-001_VALID_LOGIN_RESPONSE.png")</f>
+        <v>E2 — TC-AUTH-001_VALID_LOGIN_RESPONSE.png</v>
+      </c>
+      <c r="I16" s="21"/>
+    </row>
+    <row r="17" ht="34" customHeight="1" spans="1:9">
+      <c r="A17" s="18"/>
+      <c r="B17" s="19"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="18"/>
+      <c r="F17" s="21"/>
+      <c r="G17" s="18"/>
+      <c r="H17" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/authentication/SETUP_CREATE_AUTH_USER_REQUEST.png","SETUP — Create User Request")</f>
+        <v>SETUP — Create User Request</v>
+      </c>
+      <c r="I17" s="21"/>
+    </row>
+    <row r="18" ht="34" customHeight="1" spans="1:9">
+      <c r="A18" s="18"/>
+      <c r="B18" s="19"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="18"/>
+      <c r="H18" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/authentication/SETUP_CREATE_AUTH_USER_RESPONSE.png","SETUP — Create User Response")</f>
+        <v>SETUP — Create User Response</v>
+      </c>
+      <c r="I18" s="21"/>
+    </row>
+    <row r="19" ht="34" customHeight="1" spans="1:9">
+      <c r="A19" s="23" t="s">
+        <v>177</v>
+      </c>
+      <c r="B19" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="C19" s="25">
+        <v>46314</v>
+      </c>
+      <c r="D19" s="24" t="s">
+        <v>161</v>
+      </c>
+      <c r="E19" s="23">
+        <v>401</v>
+      </c>
+      <c r="F19" s="26" t="s">
+        <v>178</v>
+      </c>
+      <c r="G19" s="23" t="s">
+        <v>163</v>
+      </c>
+      <c r="H19" s="27" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/authentication/TC-AUTH-002_INVALID_PASSWORD_REQUEST.png","E1 — TC-AUTH-002_INVALID_PASSWORD_REQUEST.png")</f>
+        <v>E1 — TC-AUTH-002_INVALID_PASSWORD_REQUEST.png</v>
+      </c>
+      <c r="I19" s="26" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1" spans="1:9">
+      <c r="A20" s="23"/>
+      <c r="B20" s="24"/>
+      <c r="C20" s="25"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="23"/>
+      <c r="F20" s="26"/>
+      <c r="G20" s="23"/>
+      <c r="H20" s="27" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/authentication/TC-AUTH-002_INVALID_PASSWORD_RESPONSE.png","E2 — TC-AUTH-002_INVALID_PASSWORD_RESPONSE.png")</f>
+        <v>E2 — TC-AUTH-002_INVALID_PASSWORD_RESPONSE.png</v>
+      </c>
+      <c r="I20" s="26"/>
+    </row>
+    <row r="21" ht="34" customHeight="1" spans="1:9">
+      <c r="A21" s="18" t="s">
+        <v>180</v>
+      </c>
+      <c r="B21" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="C21" s="20">
+        <v>46314</v>
+      </c>
+      <c r="D21" s="19" t="s">
+        <v>161</v>
+      </c>
+      <c r="E21" s="18">
+        <v>401</v>
+      </c>
+      <c r="F21" s="21" t="s">
+        <v>181</v>
+      </c>
+      <c r="G21" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="H21" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/authentication/TC-AUTH-003_UNREGISTERED_EMAIL_REQUEST.png","E1 — TC-AUTH-003_UNREGISTERED_EMAIL_REQUEST.png")</f>
+        <v>E1 — TC-AUTH-003_UNREGISTERED_EMAIL_REQUEST.png</v>
+      </c>
+      <c r="I21" s="21" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1" spans="1:9">
+      <c r="A22" s="18"/>
+      <c r="B22" s="19"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="18"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="18"/>
+      <c r="H22" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/authentication/TC-AUTH-003_UNREGISTERED_EMAIL_RESPONSE.png","E2 — TC-AUTH-003_UNREGISTERED_EMAIL_RESPONSE.png")</f>
+        <v>E2 — TC-AUTH-003_UNREGISTERED_EMAIL_RESPONSE.png</v>
+      </c>
+      <c r="I22" s="21"/>
+    </row>
+    <row r="23" ht="34" customHeight="1" spans="1:9">
+      <c r="A23" s="18"/>
+      <c r="B23" s="19"/>
+      <c r="C23" s="20"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="18"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="18"/>
+      <c r="H23" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/authentication/CHECK_UNREGISTERED_EMAIL_RESPONSE.png","E3 — CHECK_UNREGISTERED_EMAIL_RESPONSE.png")</f>
+        <v>E3 — CHECK_UNREGISTERED_EMAIL_RESPONSE.png</v>
+      </c>
+      <c r="I23" s="21"/>
+    </row>
+    <row r="24" ht="34" customHeight="1" spans="1:9">
+      <c r="A24" s="23" t="s">
+        <v>183</v>
+      </c>
+      <c r="B24" s="24" t="s">
+        <v>78</v>
+      </c>
+      <c r="C24" s="25">
+        <v>46315</v>
+      </c>
+      <c r="D24" s="24" t="s">
+        <v>161</v>
+      </c>
+      <c r="E24" s="23">
+        <v>400</v>
+      </c>
+      <c r="F24" s="26" t="s">
+        <v>184</v>
+      </c>
+      <c r="G24" s="23" t="s">
+        <v>163</v>
+      </c>
+      <c r="H24" s="27" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/authentication/TC-AUTH-004_MISSING_EMAIL_REQUEST.png","E1 — TC-AUTH-004_MISSING_EMAIL_REQUEST.png")</f>
+        <v>E1 — TC-AUTH-004_MISSING_EMAIL_REQUEST.png</v>
+      </c>
+      <c r="I24" s="26" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="25" ht="34" customHeight="1" spans="1:9">
+      <c r="A25" s="23"/>
+      <c r="B25" s="24"/>
+      <c r="C25" s="25"/>
+      <c r="D25" s="24"/>
+      <c r="E25" s="23"/>
+      <c r="F25" s="26"/>
+      <c r="G25" s="23"/>
+      <c r="H25" s="27" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/authentication/TC-AUTH-004_MISSING_EMAIL_RESPONSE.png","E2 — TC-AUTH-004_MISSING_EMAIL_RESPONSE.png")</f>
+        <v>E2 — TC-AUTH-004_MISSING_EMAIL_RESPONSE.png</v>
+      </c>
+      <c r="I25" s="26"/>
+    </row>
+    <row r="26" ht="34" customHeight="1" spans="1:9">
+      <c r="A26" s="18" t="s">
+        <v>186</v>
+      </c>
+      <c r="B26" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="C26" s="20">
+        <v>46315</v>
+      </c>
+      <c r="D26" s="19" t="s">
+        <v>161</v>
+      </c>
+      <c r="E26" s="18">
+        <v>200</v>
+      </c>
+      <c r="F26" s="21" t="s">
+        <v>187</v>
+      </c>
+      <c r="G26" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="H26" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/products/TC-PROD-001_GET_PRODUCTS_REQUEST.png","E1 — TC-PROD-001_GET_PRODUCTS_REQUEST.png")</f>
+        <v>E1 — TC-PROD-001_GET_PRODUCTS_REQUEST.png</v>
+      </c>
+      <c r="I26" s="21" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="27" ht="34" customHeight="1" spans="1:9">
+      <c r="A27" s="18"/>
+      <c r="B27" s="19"/>
+      <c r="C27" s="20"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="18"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="18"/>
+      <c r="H27" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/products/TC-PROD-001_GET_PRODUCTS_RESPONSE.png","E2 — TC-PROD-001_GET_PRODUCTS_RESPONSE.png")</f>
+        <v>E2 — TC-PROD-001_GET_PRODUCTS_RESPONSE.png</v>
+      </c>
+      <c r="I27" s="21"/>
+    </row>
+    <row r="28" ht="34" customHeight="1" spans="1:9">
+      <c r="A28" s="23" t="s">
+        <v>189</v>
+      </c>
+      <c r="B28" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="C28" s="25">
+        <v>46316</v>
+      </c>
+      <c r="D28" s="24" t="s">
+        <v>161</v>
+      </c>
+      <c r="E28" s="23">
+        <v>200</v>
+      </c>
+      <c r="F28" s="26" t="s">
+        <v>190</v>
+      </c>
+      <c r="G28" s="23" t="s">
+        <v>163</v>
+      </c>
+      <c r="H28" s="27" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/products/TC-PROD-002_GET_PRODUCT_REQUEST.png","E1 — TC-PROD-002_GET_PRODUCT_REQUEST.png")</f>
+        <v>E1 — TC-PROD-002_GET_PRODUCT_REQUEST.png</v>
+      </c>
+      <c r="I28" s="26" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="29" ht="34" customHeight="1" spans="1:9">
+      <c r="A29" s="23"/>
+      <c r="B29" s="24"/>
+      <c r="C29" s="25"/>
+      <c r="D29" s="24"/>
+      <c r="E29" s="23"/>
+      <c r="F29" s="26"/>
+      <c r="G29" s="23"/>
+      <c r="H29" s="27" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/products/TC-PROD-002_GET_PRODUCT_RESPONSE.png","E2 — TC-PROD-002_GET_PRODUCT_RESPONSE.png")</f>
+        <v>E2 — TC-PROD-002_GET_PRODUCT_RESPONSE.png</v>
+      </c>
+      <c r="I29" s="26"/>
+    </row>
+    <row r="30" ht="34" customHeight="1" spans="1:9">
+      <c r="A30" s="18" t="s">
+        <v>192</v>
+      </c>
+      <c r="B30" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="C30" s="20">
+        <v>46318</v>
+      </c>
+      <c r="D30" s="19" t="s">
+        <v>161</v>
+      </c>
+      <c r="E30" s="18">
+        <v>201</v>
+      </c>
+      <c r="F30" s="21" t="s">
+        <v>193</v>
+      </c>
+      <c r="G30" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="H30" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/products/TC-PROD-003_CREATE_PRODUCT_REQUEST.png","E1 — TC-PROD-003_CREATE_PRODUCT_REQUEST.png")</f>
+        <v>E1 — TC-PROD-003_CREATE_PRODUCT_REQUEST.png</v>
+      </c>
+      <c r="I30" s="21" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="31" ht="34" customHeight="1" spans="1:9">
+      <c r="A31" s="18"/>
+      <c r="B31" s="19"/>
+      <c r="C31" s="20"/>
+      <c r="D31" s="19"/>
+      <c r="E31" s="18"/>
+      <c r="F31" s="21"/>
+      <c r="G31" s="18"/>
+      <c r="H31" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/products/TC-PROD-003_CREATE_PRODUCT_RESPONSE.png","E2 — TC-PROD-003_CREATE_PRODUCT_RESPONSE.png")</f>
+        <v>E2 — TC-PROD-003_CREATE_PRODUCT_RESPONSE.png</v>
+      </c>
+      <c r="I31" s="21"/>
+    </row>
+    <row r="32" ht="34" customHeight="1" spans="1:9">
+      <c r="A32" s="18"/>
+      <c r="B32" s="19"/>
+      <c r="C32" s="20"/>
+      <c r="D32" s="19"/>
+      <c r="E32" s="18"/>
+      <c r="F32" s="21"/>
+      <c r="G32" s="18"/>
+      <c r="H32" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/products/CHECK_CREATED_PRODUCT_RESPONSE.png","E3 — CHECK_CREATED_PRODUCT_RESPONSE.png")</f>
+        <v>E3 — CHECK_CREATED_PRODUCT_RESPONSE.png</v>
+      </c>
+      <c r="I32" s="21"/>
+    </row>
+    <row r="33" ht="34" customHeight="1" spans="1:9">
+      <c r="A33" s="23" t="s">
+        <v>195</v>
+      </c>
+      <c r="B33" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="C33" s="25">
+        <v>46319</v>
+      </c>
+      <c r="D33" s="24" t="s">
+        <v>161</v>
+      </c>
+      <c r="E33" s="23">
+        <v>400</v>
+      </c>
+      <c r="F33" s="26" t="s">
         <v>196</v>
       </c>
-      <c r="I15" s="21" t="s">
+      <c r="G33" s="23" t="s">
+        <v>163</v>
+      </c>
+      <c r="H33" s="27" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/products/TC-PROD-004_DUPLICATE_PRODUCT_REQUEST.png","E1 — TC-PROD-004_DUPLICATE_PRODUCT_REQUEST.png")</f>
+        <v>E1 — TC-PROD-004_DUPLICATE_PRODUCT_REQUEST.png</v>
+      </c>
+      <c r="I33" s="26" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="16" ht="118" customHeight="1" spans="1:1024 1025:16384">
-      <c r="A16" s="23" t="s">
+    <row r="34" ht="34" customHeight="1" spans="1:9">
+      <c r="A34" s="23"/>
+      <c r="B34" s="24"/>
+      <c r="C34" s="25"/>
+      <c r="D34" s="24"/>
+      <c r="E34" s="23"/>
+      <c r="F34" s="26"/>
+      <c r="G34" s="23"/>
+      <c r="H34" s="27" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/products/TC-PROD-004_DUPLICATE_PRODUCT_RESPONSE.png","E2 — TC-PROD-004_DUPLICATE_PRODUCT_RESPONSE.png")</f>
+        <v>E2 — TC-PROD-004_DUPLICATE_PRODUCT_RESPONSE.png</v>
+      </c>
+      <c r="I34" s="26"/>
+    </row>
+    <row r="35" ht="34" customHeight="1" spans="1:9">
+      <c r="A35" s="23"/>
+      <c r="B35" s="24"/>
+      <c r="C35" s="25"/>
+      <c r="D35" s="24"/>
+      <c r="E35" s="23"/>
+      <c r="F35" s="26"/>
+      <c r="G35" s="23"/>
+      <c r="H35" s="27" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/products/TC-PROD-004_VERIFY_NO_DUPLICATE_RESPONSE.png","E3 — TC-PROD-004_VERIFY_NO_DUPLICATE_RESPONSE.png")</f>
+        <v>E3 — TC-PROD-004_VERIFY_NO_DUPLICATE_RESPONSE.png</v>
+      </c>
+      <c r="I35" s="26"/>
+    </row>
+    <row r="36" ht="34" customHeight="1" spans="1:9">
+      <c r="A36" s="18" t="s">
         <v>198</v>
       </c>
-      <c r="B16" s="23" t="s">
-        <v>93</v>
-      </c>
-      <c r="C16" s="24">
-        <v>46316</v>
-      </c>
-      <c r="D16" s="25" t="s">
+      <c r="B36" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="C36" s="20">
+        <v>46319</v>
+      </c>
+      <c r="D36" s="19" t="s">
         <v>161</v>
       </c>
-      <c r="E16" s="23">
+      <c r="E36" s="18">
+        <v>201</v>
+      </c>
+      <c r="F36" s="21" t="s">
+        <v>199</v>
+      </c>
+      <c r="G36" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="H36" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/cart/TC-CART-001_CREATE_CART_REQUEST.png","E1 — TC-CART-001_CREATE_CART_REQUEST.png")</f>
+        <v>E1 — TC-CART-001_CREATE_CART_REQUEST.png</v>
+      </c>
+      <c r="I36" s="21" t="s">
         <v>200</v>
       </c>
-      <c r="F16" s="26" t="s">
-        <v>199</v>
-      </c>
-      <c r="G16" s="23" t="s">
+    </row>
+    <row r="37" ht="34" customHeight="1" spans="1:9">
+      <c r="A37" s="18"/>
+      <c r="B37" s="19"/>
+      <c r="C37" s="20"/>
+      <c r="D37" s="19"/>
+      <c r="E37" s="18"/>
+      <c r="F37" s="21"/>
+      <c r="G37" s="18"/>
+      <c r="H37" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/cart/TC-CART-001_CREATE_CART_RESPONSE.png","E2 — TC-CART-001_CREATE_CART_RESPONSE.png")</f>
+        <v>E2 — TC-CART-001_CREATE_CART_RESPONSE.png</v>
+      </c>
+      <c r="I37" s="21"/>
+    </row>
+    <row r="38" ht="34" customHeight="1" spans="1:9">
+      <c r="A38" s="18"/>
+      <c r="B38" s="19"/>
+      <c r="C38" s="20"/>
+      <c r="D38" s="19"/>
+      <c r="E38" s="18"/>
+      <c r="F38" s="21"/>
+      <c r="G38" s="18"/>
+      <c r="H38" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/cart/TC-CART-001_VERIFY_CART_RESPONSE.png","E3 — TC-CART-001_VERIFY_CART_RESPONSE.png")</f>
+        <v>E3 — TC-CART-001_VERIFY_CART_RESPONSE.png</v>
+      </c>
+      <c r="I38" s="21"/>
+    </row>
+    <row r="39" ht="34" customHeight="1" spans="1:9">
+      <c r="A39" s="18"/>
+      <c r="B39" s="19"/>
+      <c r="C39" s="20"/>
+      <c r="D39" s="19"/>
+      <c r="E39" s="18"/>
+      <c r="F39" s="21"/>
+      <c r="G39" s="18"/>
+      <c r="H39" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/cart/TC-CART-001_STOCK_BEFORE.png","E4 — TC-CART-001_STOCK_BEFORE.png")</f>
+        <v>E4 — TC-CART-001_STOCK_BEFORE.png</v>
+      </c>
+      <c r="I39" s="21"/>
+    </row>
+    <row r="40" ht="34" customHeight="1" spans="1:9">
+      <c r="A40" s="18"/>
+      <c r="B40" s="19"/>
+      <c r="C40" s="20"/>
+      <c r="D40" s="19"/>
+      <c r="E40" s="18"/>
+      <c r="F40" s="21"/>
+      <c r="G40" s="18"/>
+      <c r="H40" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/cart/TC-CART-001_STOCK_AFTER.png","E5 — TC-CART-001_STOCK_AFTER.png")</f>
+        <v>E5 — TC-CART-001_STOCK_AFTER.png</v>
+      </c>
+      <c r="I40" s="21"/>
+    </row>
+    <row r="41" ht="34" customHeight="1" spans="1:9">
+      <c r="A41" s="23" t="s">
+        <v>201</v>
+      </c>
+      <c r="B41" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="C41" s="25">
+        <v>46319</v>
+      </c>
+      <c r="D41" s="24" t="s">
+        <v>161</v>
+      </c>
+      <c r="E41" s="23">
+        <v>400</v>
+      </c>
+      <c r="F41" s="26" t="s">
+        <v>202</v>
+      </c>
+      <c r="G41" s="23" t="s">
         <v>163</v>
       </c>
-      <c r="H16" s="27" t="s">
-        <v>200</v>
-      </c>
-      <c r="I16" s="26" t="s">
-        <v>201</v>
+      <c r="H41" s="27" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/cart/TC-CART-002_EXISTING_CART_RESPONSE.png","E1 — TC-CART-002_EXISTING_CART_RESPONSE.png")</f>
+        <v>E1 — TC-CART-002_EXISTING_CART_RESPONSE.png</v>
+      </c>
+      <c r="I41" s="26" t="s">
+        <v>203</v>
       </c>
     </row>
-    <row r="17" ht="115" customHeight="1" spans="1:9">
-      <c r="A17" s="28" t="s">
-        <v>202</v>
-      </c>
-      <c r="B17" s="28" t="s">
-        <v>101</v>
-      </c>
-      <c r="C17" s="29">
-        <v>46318</v>
-      </c>
-      <c r="D17" s="30" t="s">
+    <row r="42" ht="34" customHeight="1" spans="1:9">
+      <c r="A42" s="23"/>
+      <c r="B42" s="24"/>
+      <c r="C42" s="25"/>
+      <c r="D42" s="24"/>
+      <c r="E42" s="23"/>
+      <c r="F42" s="26"/>
+      <c r="G42" s="23"/>
+      <c r="H42" s="27" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/cart/TC-CART-002_SECOND_CART_REQUEST.png","E2 — TC-CART-002_SECOND_CART_REQUEST.png")</f>
+        <v>E2 — TC-CART-002_SECOND_CART_REQUEST.png</v>
+      </c>
+      <c r="I42" s="26"/>
+    </row>
+    <row r="43" ht="34" customHeight="1" spans="1:9">
+      <c r="A43" s="23"/>
+      <c r="B43" s="24"/>
+      <c r="C43" s="25"/>
+      <c r="D43" s="24"/>
+      <c r="E43" s="23"/>
+      <c r="F43" s="26"/>
+      <c r="G43" s="23"/>
+      <c r="H43" s="27" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/cart/TC-CART-002_SECOND_CART_RESPONSE.png","E3 — TC-CART-002_SECOND_CART_RESPONSE.png")</f>
+        <v>E3 — TC-CART-002_SECOND_CART_RESPONSE.png</v>
+      </c>
+      <c r="I43" s="26"/>
+    </row>
+    <row r="44" ht="34" customHeight="1" spans="1:9">
+      <c r="A44" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="B44" s="19" t="s">
+        <v>131</v>
+      </c>
+      <c r="C44" s="20">
+        <v>46320</v>
+      </c>
+      <c r="D44" s="19" t="s">
         <v>161</v>
       </c>
-      <c r="E17" s="28">
-        <v>201</v>
-      </c>
-      <c r="F17" s="31" t="s">
-        <v>203</v>
-      </c>
-      <c r="G17" s="28" t="s">
+      <c r="E44" s="18">
+        <v>400</v>
+      </c>
+      <c r="F44" s="21" t="s">
+        <v>205</v>
+      </c>
+      <c r="G44" s="18" t="s">
         <v>163</v>
       </c>
-      <c r="H17" s="32" t="s">
-        <v>204</v>
-      </c>
-      <c r="I17" s="31" t="s">
-        <v>205</v>
+      <c r="H44" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/cart/TC-CART-003_STOCK_BEFORE.png","E1 — TC-CART-003_STOCK_BEFORE.png")</f>
+        <v>E1 — TC-CART-003_STOCK_BEFORE.png</v>
+      </c>
+      <c r="I44" s="21" t="s">
+        <v>206</v>
       </c>
     </row>
-    <row r="18" ht="95" customHeight="1" spans="1:9">
-      <c r="A18" s="23" t="s">
-        <v>206</v>
-      </c>
-      <c r="B18" s="23" t="s">
-        <v>108</v>
-      </c>
-      <c r="C18" s="24">
-        <v>46319</v>
-      </c>
-      <c r="D18" s="25" t="s">
+    <row r="45" ht="34" customHeight="1" spans="1:9">
+      <c r="A45" s="18"/>
+      <c r="B45" s="19"/>
+      <c r="C45" s="20"/>
+      <c r="D45" s="19"/>
+      <c r="E45" s="18"/>
+      <c r="F45" s="21"/>
+      <c r="G45" s="18"/>
+      <c r="H45" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/cart/TC-CART-003_INSUFFICIENT_STOCK_REQUEST.png","E2 — TC-CART-003_INSUFFICIENT_STOCK_REQUEST.png")</f>
+        <v>E2 — TC-CART-003_INSUFFICIENT_STOCK_REQUEST.png</v>
+      </c>
+      <c r="I45" s="21"/>
+    </row>
+    <row r="46" ht="34" customHeight="1" spans="1:9">
+      <c r="A46" s="18"/>
+      <c r="B46" s="19"/>
+      <c r="C46" s="20"/>
+      <c r="D46" s="19"/>
+      <c r="E46" s="18"/>
+      <c r="F46" s="21"/>
+      <c r="G46" s="18"/>
+      <c r="H46" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/cart/TC-CART-003_INSUFFICIENT_STOCK_RESPONSE.png","E3 — TC-CART-003_INSUFFICIENT_STOCK_RESPONSE.png")</f>
+        <v>E3 — TC-CART-003_INSUFFICIENT_STOCK_RESPONSE.png</v>
+      </c>
+      <c r="I46" s="21"/>
+    </row>
+    <row r="47" ht="34" customHeight="1" spans="1:9">
+      <c r="A47" s="18"/>
+      <c r="B47" s="19"/>
+      <c r="C47" s="20"/>
+      <c r="D47" s="19"/>
+      <c r="E47" s="18"/>
+      <c r="F47" s="21"/>
+      <c r="G47" s="18"/>
+      <c r="H47" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/cart/TC-CART-003_STOCK_AFTER.png","E4 — TC-CART-003_STOCK_AFTER.png")</f>
+        <v>E4 — TC-CART-003_STOCK_AFTER.png</v>
+      </c>
+      <c r="I47" s="21"/>
+    </row>
+    <row r="48" ht="34" customHeight="1" spans="1:9">
+      <c r="A48" s="18"/>
+      <c r="B48" s="19"/>
+      <c r="C48" s="20"/>
+      <c r="D48" s="19"/>
+      <c r="E48" s="18"/>
+      <c r="F48" s="21"/>
+      <c r="G48" s="18"/>
+      <c r="H48" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/cart/TC-CART-003_VERIFY_NO_CART_RESPONSE.png","E5 — TC-CART-003_VERIFY_NO_CART_RESPONSE.png")</f>
+        <v>E5 — TC-CART-003_VERIFY_NO_CART_RESPONSE.png</v>
+      </c>
+      <c r="I48" s="21"/>
+    </row>
+    <row r="49" ht="34" customHeight="1" spans="1:9">
+      <c r="A49" s="18"/>
+      <c r="B49" s="19"/>
+      <c r="C49" s="20"/>
+      <c r="D49" s="19"/>
+      <c r="E49" s="18"/>
+      <c r="F49" s="21"/>
+      <c r="G49" s="18"/>
+      <c r="H49" s="22" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/cart/TC-CART-003_USER_SETUP_RESPONSE.png","SETUP — User Response")</f>
+        <v>SETUP — User Response</v>
+      </c>
+      <c r="I49" s="21"/>
+    </row>
+    <row r="50" ht="34" customHeight="1" spans="1:9">
+      <c r="A50" s="23" t="s">
+        <v>207</v>
+      </c>
+      <c r="B50" s="24" t="s">
+        <v>138</v>
+      </c>
+      <c r="C50" s="25">
+        <v>46320</v>
+      </c>
+      <c r="D50" s="24" t="s">
         <v>161</v>
       </c>
-      <c r="E18" s="23">
+      <c r="E50" s="23">
         <v>400</v>
       </c>
-      <c r="F18" s="26" t="s">
-        <v>207</v>
-      </c>
-      <c r="G18" s="23" t="s">
+      <c r="F50" s="26" t="s">
+        <v>208</v>
+      </c>
+      <c r="G50" s="23" t="s">
         <v>163</v>
       </c>
-      <c r="H18" s="27" t="s">
-        <v>208</v>
-      </c>
-      <c r="I18" s="26" t="s">
+      <c r="H50" s="27" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/cart/TC-CART-004_INVALID_PRODUCT_CHECK.png","E1 — TC-CART-004_INVALID_PRODUCT_CHECK.png")</f>
+        <v>E1 — TC-CART-004_INVALID_PRODUCT_CHECK.png</v>
+      </c>
+      <c r="I50" s="26" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="19" ht="113" customHeight="1" spans="1:9">
-      <c r="A19" s="28" t="s">
-        <v>210</v>
-      </c>
-      <c r="B19" s="28" t="s">
-        <v>115</v>
-      </c>
-      <c r="C19" s="29">
-        <v>46319</v>
-      </c>
-      <c r="D19" s="30" t="s">
-        <v>161</v>
-      </c>
-      <c r="E19" s="28">
-        <v>201</v>
-      </c>
-      <c r="F19" s="31" t="s">
-        <v>211</v>
-      </c>
-      <c r="G19" s="28" t="s">
-        <v>163</v>
-      </c>
-      <c r="H19" s="32" t="s">
-        <v>212</v>
-      </c>
-      <c r="I19" s="31" t="s">
-        <v>213</v>
-      </c>
+    <row r="51" ht="34" customHeight="1" spans="1:9">
+      <c r="A51" s="23"/>
+      <c r="B51" s="24"/>
+      <c r="C51" s="25"/>
+      <c r="D51" s="24"/>
+      <c r="E51" s="23"/>
+      <c r="F51" s="26"/>
+      <c r="G51" s="23"/>
+      <c r="H51" s="27" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/cart/TC-CART-004_INVALID_PRODUCT_REQUEST.png","E2 — TC-CART-004_INVALID_PRODUCT_REQUEST.png")</f>
+        <v>E2 — TC-CART-004_INVALID_PRODUCT_REQUEST.png</v>
+      </c>
+      <c r="I51" s="26"/>
     </row>
-    <row r="20" ht="90" customHeight="1" spans="1:9">
-      <c r="A20" s="33" t="s">
-        <v>214</v>
-      </c>
-      <c r="B20" s="33" t="s">
-        <v>124</v>
-      </c>
-      <c r="C20" s="34">
-        <v>46319</v>
-      </c>
-      <c r="D20" s="35" t="s">
-        <v>161</v>
-      </c>
-      <c r="E20" s="33">
-        <v>400</v>
-      </c>
-      <c r="F20" s="36" t="s">
-        <v>215</v>
-      </c>
-      <c r="G20" s="33" t="s">
-        <v>163</v>
-      </c>
-      <c r="H20" s="37" t="s">
-        <v>216</v>
-      </c>
-      <c r="I20" s="36" t="s">
-        <v>217</v>
-      </c>
+    <row r="52" ht="34" customHeight="1" spans="1:9">
+      <c r="A52" s="23"/>
+      <c r="B52" s="24"/>
+      <c r="C52" s="25"/>
+      <c r="D52" s="24"/>
+      <c r="E52" s="23"/>
+      <c r="F52" s="26"/>
+      <c r="G52" s="23"/>
+      <c r="H52" s="27" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/cart/TC-CART-004_INVALID_PRODUCT_RESPONSE.png","E3 — TC-CART-004_INVALID_PRODUCT_RESPONSE.png")</f>
+        <v>E3 — TC-CART-004_INVALID_PRODUCT_RESPONSE.png</v>
+      </c>
+      <c r="I52" s="26"/>
     </row>
-    <row r="21" ht="171" customHeight="1" spans="1:9">
-      <c r="A21" s="28" t="s">
-        <v>218</v>
-      </c>
-      <c r="B21" s="28" t="s">
-        <v>131</v>
-      </c>
-      <c r="C21" s="29">
-        <v>46320</v>
-      </c>
-      <c r="D21" s="30" t="s">
-        <v>161</v>
-      </c>
-      <c r="E21" s="28">
-        <v>400</v>
-      </c>
-      <c r="F21" s="31" t="s">
-        <v>219</v>
-      </c>
-      <c r="G21" s="28" t="s">
-        <v>163</v>
-      </c>
-      <c r="H21" s="32" t="s">
-        <v>220</v>
-      </c>
-      <c r="I21" s="31" t="s">
-        <v>221</v>
-      </c>
+    <row r="53" ht="34" customHeight="1" spans="1:9">
+      <c r="A53" s="23"/>
+      <c r="B53" s="24"/>
+      <c r="C53" s="25"/>
+      <c r="D53" s="24"/>
+      <c r="E53" s="23"/>
+      <c r="F53" s="26"/>
+      <c r="G53" s="23"/>
+      <c r="H53" s="27" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/cart/TC-CART-004_VERIFY_NO_CART_RESPONSE.png","E4 — TC-CART-004_VERIFY_NO_CART_RESPONSE.png")</f>
+        <v>E4 — TC-CART-004_VERIFY_NO_CART_RESPONSE.png</v>
+      </c>
+      <c r="I53" s="26"/>
     </row>
-    <row r="22" ht="152" customHeight="1" spans="1:9">
-      <c r="A22" s="23" t="s">
-        <v>222</v>
-      </c>
-      <c r="B22" s="23" t="s">
-        <v>138</v>
-      </c>
-      <c r="C22" s="24">
-        <v>46320</v>
-      </c>
-      <c r="D22" s="25" t="s">
-        <v>161</v>
-      </c>
-      <c r="E22" s="23">
-        <v>400</v>
-      </c>
-      <c r="F22" s="26" t="s">
-        <v>223</v>
-      </c>
-      <c r="G22" s="23" t="s">
-        <v>163</v>
-      </c>
-      <c r="H22" s="27" t="s">
-        <v>224</v>
-      </c>
-      <c r="I22" s="26" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="23" ht="58" customHeight="1" spans="1:9">
-      <c r="A23" s="38"/>
-      <c r="B23" s="38"/>
-      <c r="C23" s="39"/>
-      <c r="D23" s="40"/>
-      <c r="E23" s="38"/>
-      <c r="F23" s="40"/>
-      <c r="G23" s="40"/>
-      <c r="H23" s="41"/>
-      <c r="I23" s="40"/>
-    </row>
-    <row r="24" ht="58" customHeight="1" spans="1:9">
-      <c r="A24" s="42"/>
-      <c r="B24" s="42"/>
-      <c r="C24" s="43"/>
-      <c r="D24" s="44"/>
-      <c r="E24" s="42"/>
-      <c r="F24" s="44"/>
-      <c r="G24" s="44"/>
-      <c r="H24" s="45"/>
-      <c r="I24" s="44"/>
-    </row>
-    <row r="25" ht="58" customHeight="1" spans="1:9">
-      <c r="A25" s="46"/>
-      <c r="B25" s="46"/>
-      <c r="C25" s="47"/>
-      <c r="D25" s="48"/>
-      <c r="E25" s="46"/>
-      <c r="F25" s="48"/>
-      <c r="G25" s="48"/>
-      <c r="H25" s="49"/>
-      <c r="I25" s="48"/>
-    </row>
-    <row r="26" ht="58" customHeight="1" spans="1:9">
-      <c r="A26" s="42"/>
-      <c r="B26" s="42"/>
-      <c r="C26" s="43"/>
-      <c r="D26" s="44"/>
-      <c r="E26" s="42"/>
-      <c r="F26" s="44"/>
-      <c r="G26" s="44"/>
-      <c r="H26" s="45"/>
-      <c r="I26" s="44"/>
-    </row>
-    <row r="27" ht="58" customHeight="1" spans="1:9">
-      <c r="A27" s="46"/>
-      <c r="B27" s="46"/>
-      <c r="C27" s="47"/>
-      <c r="D27" s="48"/>
-      <c r="E27" s="46"/>
-      <c r="F27" s="48"/>
-      <c r="G27" s="48"/>
-      <c r="H27" s="49"/>
-      <c r="I27" s="48"/>
-    </row>
-    <row r="28" ht="58" customHeight="1" spans="1:9">
-      <c r="A28" s="42"/>
-      <c r="B28" s="42"/>
-      <c r="C28" s="43"/>
-      <c r="D28" s="44"/>
-      <c r="E28" s="42"/>
-      <c r="F28" s="44"/>
-      <c r="G28" s="44"/>
-      <c r="H28" s="45"/>
-      <c r="I28" s="44"/>
-    </row>
-    <row r="29" ht="58" customHeight="1" spans="1:9">
-      <c r="A29" s="46"/>
-      <c r="B29" s="46"/>
-      <c r="C29" s="47"/>
-      <c r="D29" s="48"/>
-      <c r="E29" s="46"/>
-      <c r="F29" s="48"/>
-      <c r="G29" s="48"/>
-      <c r="H29" s="49"/>
-      <c r="I29" s="48"/>
-    </row>
-    <row r="30" ht="58" customHeight="1" spans="1:9">
-      <c r="A30" s="42"/>
-      <c r="B30" s="42"/>
-      <c r="C30" s="43"/>
-      <c r="D30" s="44"/>
-      <c r="E30" s="42"/>
-      <c r="F30" s="44"/>
-      <c r="G30" s="44"/>
-      <c r="H30" s="45"/>
-      <c r="I30" s="44"/>
-    </row>
-    <row r="31" ht="58" customHeight="1" spans="1:9">
-      <c r="A31" s="46"/>
-      <c r="B31" s="46"/>
-      <c r="C31" s="47"/>
-      <c r="D31" s="48"/>
-      <c r="E31" s="46"/>
-      <c r="F31" s="48"/>
-      <c r="G31" s="48"/>
-      <c r="H31" s="49"/>
-      <c r="I31" s="48"/>
-    </row>
-    <row r="32" spans="1:9">
-      <c r="C32" s="50"/>
-    </row>
-    <row r="33" spans="3:3">
-      <c r="C33" s="50"/>
-    </row>
-    <row r="34" spans="3:3">
-      <c r="C34" s="50"/>
-    </row>
-    <row r="35" spans="3:3">
-      <c r="C35" s="50"/>
-    </row>
-    <row r="36" spans="3:3">
-      <c r="C36" s="50"/>
-    </row>
-    <row r="37" spans="3:3">
-      <c r="C37" s="50"/>
-    </row>
-    <row r="38" spans="3:3">
-      <c r="C38" s="50"/>
-    </row>
-    <row r="39" spans="3:3">
-      <c r="C39" s="50"/>
-    </row>
-    <row r="40" spans="3:3">
-      <c r="C40" s="50"/>
-    </row>
-    <row r="41" spans="3:3">
-      <c r="C41" s="50"/>
-    </row>
-    <row r="42" spans="3:3">
-      <c r="C42" s="50"/>
-    </row>
-    <row r="43" spans="3:3">
-      <c r="C43" s="50"/>
-    </row>
-    <row r="44" spans="3:3">
-      <c r="C44" s="50"/>
-    </row>
-    <row r="45" spans="3:3">
-      <c r="C45" s="50"/>
-    </row>
-    <row r="46" spans="3:3">
-      <c r="C46" s="50"/>
-    </row>
-    <row r="47" spans="3:3">
-      <c r="C47" s="50"/>
-    </row>
-    <row r="48" spans="3:3">
-      <c r="C48" s="50"/>
-    </row>
-    <row r="49" spans="3:3">
-      <c r="C49" s="50"/>
-    </row>
-    <row r="50" spans="3:3">
-      <c r="C50" s="50"/>
-    </row>
-    <row r="51" spans="3:3">
-      <c r="C51" s="50"/>
+    <row r="54" ht="34" customHeight="1" spans="1:9">
+      <c r="A54" s="23"/>
+      <c r="B54" s="24"/>
+      <c r="C54" s="25"/>
+      <c r="D54" s="24"/>
+      <c r="E54" s="23"/>
+      <c r="F54" s="26"/>
+      <c r="G54" s="23"/>
+      <c r="H54" s="27" t="str">
+        <f>HYPERLINK("https://github.com/kritsada-chaisongkram/serverest-api-testing/blob/main/evidence/manual-api/cart/TC-CART-004_USER_SETUP_RESPONSE.png","SETUP — User Response")</f>
+        <v>SETUP — User Response</v>
+      </c>
+      <c r="I54" s="26"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="135">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A3:I3"/>
@@ -20623,6 +20788,134 @@
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="E5:G5"/>
     <mergeCell ref="H5:I5"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="A15:A18"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A21:A23"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="A30:A32"/>
+    <mergeCell ref="A33:A35"/>
+    <mergeCell ref="A36:A40"/>
+    <mergeCell ref="A41:A43"/>
+    <mergeCell ref="A44:A49"/>
+    <mergeCell ref="A50:A54"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="B15:B18"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="B21:B23"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="B30:B32"/>
+    <mergeCell ref="B33:B35"/>
+    <mergeCell ref="B36:B40"/>
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="B44:B49"/>
+    <mergeCell ref="B50:B54"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="C15:C18"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="C21:C23"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="C28:C29"/>
+    <mergeCell ref="C30:C32"/>
+    <mergeCell ref="C33:C35"/>
+    <mergeCell ref="C36:C40"/>
+    <mergeCell ref="C41:C43"/>
+    <mergeCell ref="C44:C49"/>
+    <mergeCell ref="C50:C54"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="D15:D18"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="D21:D23"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="D28:D29"/>
+    <mergeCell ref="D30:D32"/>
+    <mergeCell ref="D33:D35"/>
+    <mergeCell ref="D36:D40"/>
+    <mergeCell ref="D41:D43"/>
+    <mergeCell ref="D44:D49"/>
+    <mergeCell ref="D50:D54"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="E15:E18"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="E21:E23"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="E26:E27"/>
+    <mergeCell ref="E28:E29"/>
+    <mergeCell ref="E30:E32"/>
+    <mergeCell ref="E33:E35"/>
+    <mergeCell ref="E36:E40"/>
+    <mergeCell ref="E41:E43"/>
+    <mergeCell ref="E44:E49"/>
+    <mergeCell ref="E50:E54"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="F15:F18"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="F21:F23"/>
+    <mergeCell ref="F24:F25"/>
+    <mergeCell ref="F26:F27"/>
+    <mergeCell ref="F28:F29"/>
+    <mergeCell ref="F30:F32"/>
+    <mergeCell ref="F33:F35"/>
+    <mergeCell ref="F36:F40"/>
+    <mergeCell ref="F41:F43"/>
+    <mergeCell ref="F44:F49"/>
+    <mergeCell ref="F50:F54"/>
+    <mergeCell ref="G7:G8"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="G13:G14"/>
+    <mergeCell ref="G15:G18"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="G21:G23"/>
+    <mergeCell ref="G24:G25"/>
+    <mergeCell ref="G26:G27"/>
+    <mergeCell ref="G28:G29"/>
+    <mergeCell ref="G30:G32"/>
+    <mergeCell ref="G33:G35"/>
+    <mergeCell ref="G36:G40"/>
+    <mergeCell ref="G41:G43"/>
+    <mergeCell ref="G44:G49"/>
+    <mergeCell ref="G50:G54"/>
+    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="I13:I14"/>
+    <mergeCell ref="I15:I18"/>
+    <mergeCell ref="I19:I20"/>
+    <mergeCell ref="I21:I23"/>
+    <mergeCell ref="I24:I25"/>
+    <mergeCell ref="I26:I27"/>
+    <mergeCell ref="I28:I29"/>
+    <mergeCell ref="I30:I32"/>
+    <mergeCell ref="I33:I35"/>
+    <mergeCell ref="I36:I40"/>
+    <mergeCell ref="I41:I43"/>
+    <mergeCell ref="I44:I49"/>
+    <mergeCell ref="I50:I54"/>
   </mergeCells>
   <conditionalFormatting sqref="G7:G51">
     <cfRule type="expression" dxfId="1" priority="1">
@@ -20645,8 +20938,5 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
</xml_diff>